<commit_message>
📅 日报更新 2026-09-06 03:05
</commit_message>
<xml_diff>
--- a/data/exports/黄老师/dist_order_2026-09-06.xlsx
+++ b/data/exports/黄老师/dist_order_2026-09-06.xlsx
@@ -125,11 +125,11 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="0">
-        <v>50100338</v>
+        <v>50116869</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>青山绿水</t>
+          <t>美义</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 23:10:04</t>
+          <t>2026-09-06 10:56:33</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -164,7 +164,7 @@
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J2" s="0" t="inlineStr">
@@ -185,11 +185,11 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="0">
-        <v>50100035</v>
+        <v>50114006</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>杨</t>
+          <t>幸运草</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -214,7 +214,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:57:53</t>
+          <t>2026-09-06 09:45:01</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -224,7 +224,7 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J3" s="0" t="inlineStr">
@@ -245,11 +245,11 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="0">
-        <v>50100033</v>
+        <v>50113664</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>雨后彩虹</t>
+          <t>执子之手</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -274,7 +274,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:57:47</t>
+          <t>2026-09-06 09:37:35</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -284,7 +284,7 @@
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J4" s="0" t="inlineStr">
@@ -305,11 +305,11 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="0">
-        <v>50100028</v>
+        <v>50113641</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>首信海报</t>
+          <t>新视野</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -334,7 +334,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:57:32</t>
+          <t>2026-09-06 09:36:52</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -344,7 +344,7 @@
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J5" s="0" t="inlineStr">
@@ -365,11 +365,11 @@
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="0">
-        <v>50099958</v>
+        <v>50113640</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>张君</t>
+          <t>安静且聆听</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -394,7 +394,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:55:57</t>
+          <t>2026-09-06 09:36:49</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -404,7 +404,7 @@
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J6" s="0" t="inlineStr">
@@ -420,16 +420,21 @@
       <c r="L6" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N6" s="0" t="inlineStr">
+        <is>
+          <t>保山</t>
         </is>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="0">
-        <v>50099933</v>
+        <v>50113638</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>耶和华以勒</t>
+          <t>十月</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -454,7 +459,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:55:31</t>
+          <t>2026-09-06 09:36:45</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -464,7 +469,7 @@
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J7" s="0" t="inlineStr">
@@ -485,11 +490,11 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="0">
-        <v>50099844</v>
+        <v>50100338</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>平安</t>
+          <t>青山绿水</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -514,7 +519,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:51:49</t>
+          <t>2026-09-05 23:10:04</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -524,7 +529,7 @@
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J8" s="0" t="inlineStr">
@@ -545,11 +550,11 @@
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="0">
-        <v>50099768</v>
+        <v>50100035</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>阳</t>
+          <t>杨</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -574,7 +579,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:49:01</t>
+          <t>2026-09-05 22:57:53</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -584,7 +589,7 @@
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J9" s="0" t="inlineStr">
@@ -605,11 +610,11 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="0">
-        <v>50099767</v>
+        <v>50100033</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>梦&amp;爷💫</t>
+          <t>雨后彩虹</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -634,7 +639,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:57</t>
+          <t>2026-09-05 22:57:47</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
@@ -644,7 +649,7 @@
       </c>
       <c r="I10" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J10" s="0" t="inlineStr">
@@ -665,11 +670,11 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="0">
-        <v>50099763</v>
+        <v>50100028</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>李丽</t>
+          <t>首信海报</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -694,7 +699,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:53</t>
+          <t>2026-09-05 22:57:32</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -704,7 +709,7 @@
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J11" s="0" t="inlineStr">
@@ -725,11 +730,11 @@
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="0">
-        <v>50099760</v>
+        <v>50099958</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>A选择无悔</t>
+          <t>张君</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -754,7 +759,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:46</t>
+          <t>2026-09-05 22:55:57</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -764,7 +769,7 @@
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
@@ -785,11 +790,11 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="0">
-        <v>50099759</v>
+        <v>50099933</v>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>信念</t>
+          <t>耶和华以勒</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -814,7 +819,7 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:44</t>
+          <t>2026-09-05 22:55:31</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
@@ -824,7 +829,7 @@
       </c>
       <c r="I13" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J13" s="0" t="inlineStr">
@@ -845,11 +850,11 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="0">
-        <v>50099757</v>
+        <v>50099844</v>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>李lee</t>
+          <t>平安</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -874,7 +879,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:41</t>
+          <t>2026-09-05 22:51:49</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -884,7 +889,7 @@
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
@@ -905,11 +910,11 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="0">
-        <v>50099755</v>
+        <v>50099768</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>徐飛燕*^O^*</t>
+          <t>阳</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -934,7 +939,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:39</t>
+          <t>2026-09-05 22:49:01</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -965,11 +970,11 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="0">
-        <v>50099752</v>
+        <v>50099767</v>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>星移*</t>
+          <t>梦&amp;爷💫</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -994,7 +999,7 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:35</t>
+          <t>2026-09-05 22:48:57</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
@@ -1025,11 +1030,11 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="0">
-        <v>50099749</v>
+        <v>50099763</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>刘勇</t>
+          <t>李丽</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1054,7 +1059,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:28</t>
+          <t>2026-09-05 22:48:53</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
@@ -1085,11 +1090,11 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="0">
-        <v>50099741</v>
+        <v>50099760</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>碧皓之游</t>
+          <t>A选择无悔</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -1114,7 +1119,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:15</t>
+          <t>2026-09-05 22:48:46</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
@@ -1145,11 +1150,11 @@
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="0">
-        <v>50099737</v>
+        <v>50099759</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>书心燕语</t>
+          <t>信念</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -1174,7 +1179,7 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:03</t>
+          <t>2026-09-05 22:48:44</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
@@ -1205,11 +1210,11 @@
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="0">
-        <v>50099733</v>
+        <v>50099757</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>ღ᭄ꦿ微微一笑ღ᭄ꦿ</t>
+          <t>李lee</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -1234,7 +1239,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:47:47</t>
+          <t>2026-09-05 22:48:41</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
@@ -1265,11 +1270,11 @@
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="0">
-        <v>50080657</v>
+        <v>50099755</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>平红</t>
+          <t>徐飛燕*^O^*</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -1294,7 +1299,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:07:13</t>
+          <t>2026-09-05 22:48:39</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
@@ -1325,11 +1330,11 @@
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="0">
-        <v>50080582</v>
+        <v>50099752</v>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>aabb</t>
+          <t>星移*</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -1354,7 +1359,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:05:19</t>
+          <t>2026-09-05 22:48:35</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
@@ -1385,11 +1390,11 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="0">
-        <v>50080559</v>
+        <v>50099749</v>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>自由人</t>
+          <t>刘勇</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -1414,7 +1419,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:04:28</t>
+          <t>2026-09-05 22:48:28</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
@@ -1445,11 +1450,11 @@
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="0">
-        <v>50080553</v>
+        <v>50099741</v>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>晶晶</t>
+          <t>碧皓之游</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -1474,7 +1479,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:04:15</t>
+          <t>2026-09-05 22:48:15</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -1505,11 +1510,11 @@
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="0">
-        <v>50080549</v>
+        <v>50099737</v>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>abc</t>
+          <t>书心燕语</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -1534,7 +1539,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:04:09</t>
+          <t>2026-09-05 22:48:03</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
@@ -1565,11 +1570,11 @@
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="0">
-        <v>50080548</v>
+        <v>50099733</v>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>盘子</t>
+          <t>ღ᭄ꦿ微微一笑ღ᭄ꦿ</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -1594,7 +1599,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:04:08</t>
+          <t>2026-09-05 22:47:47</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -1625,11 +1630,11 @@
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="0">
-        <v>50080547</v>
+        <v>50080657</v>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>赵满珍C5</t>
+          <t>平红</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1654,7 +1659,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:04:05</t>
+          <t>2026-09-05 13:07:13</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
@@ -1685,11 +1690,11 @@
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="0">
-        <v>50080539</v>
+        <v>50080582</v>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>平平安安</t>
+          <t>aabb</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -1714,7 +1719,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:51</t>
+          <t>2026-09-05 13:05:19</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
@@ -1745,11 +1750,11 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" s="0">
-        <v>50080538</v>
+        <v>50080559</v>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>凡事包容</t>
+          <t>自由人</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -1774,7 +1779,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:51</t>
+          <t>2026-09-05 13:04:28</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
@@ -1805,11 +1810,11 @@
     </row>
     <row r="30" spans="1:14">
       <c r="A30" s="0">
-        <v>50080536</v>
+        <v>50080553</v>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>吴忧无忧</t>
+          <t>晶晶</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -1834,7 +1839,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:47</t>
+          <t>2026-09-05 13:04:15</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
@@ -1865,11 +1870,11 @@
     </row>
     <row r="31" spans="1:14">
       <c r="A31" s="0">
-        <v>50080535</v>
+        <v>50080549</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>小鱼儿</t>
+          <t>abc</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -1894,7 +1899,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:43</t>
+          <t>2026-09-05 13:04:09</t>
         </is>
       </c>
       <c r="H31" s="0" t="inlineStr">
@@ -1925,11 +1930,11 @@
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="0">
-        <v>50080525</v>
+        <v>50080548</v>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>辞芝锦😎</t>
+          <t>盘子</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -1954,7 +1959,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:29</t>
+          <t>2026-09-05 13:04:08</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -1985,11 +1990,11 @@
     </row>
     <row r="33" spans="1:14">
       <c r="A33" s="0">
-        <v>50080523</v>
+        <v>50080547</v>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>早陈</t>
+          <t>赵满珍C5</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2014,7 +2019,7 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:21</t>
+          <t>2026-09-05 13:04:05</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
@@ -2045,11 +2050,11 @@
     </row>
     <row r="34" spans="1:14">
       <c r="A34" s="0">
-        <v>50080516</v>
+        <v>50080539</v>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>星星の恋人</t>
+          <t>平平安安</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -2074,7 +2079,7 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:13</t>
+          <t>2026-09-05 13:03:51</t>
         </is>
       </c>
       <c r="H34" s="0" t="inlineStr">
@@ -2105,11 +2110,11 @@
     </row>
     <row r="35" spans="1:14">
       <c r="A35" s="0">
-        <v>50080511</v>
+        <v>50080538</v>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>无咎</t>
+          <t>凡事包容</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -2134,7 +2139,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:09</t>
+          <t>2026-09-05 13:03:51</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
@@ -2165,11 +2170,11 @@
     </row>
     <row r="36" spans="1:14">
       <c r="A36" s="0">
-        <v>50080477</v>
+        <v>50080536</v>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>刘小虎</t>
+          <t>吴忧无忧</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -2194,7 +2199,7 @@
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:02:37</t>
+          <t>2026-09-05 13:03:47</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
@@ -2225,11 +2230,11 @@
     </row>
     <row r="37" spans="1:14">
       <c r="A37" s="0">
-        <v>50074867</v>
+        <v>50080535</v>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>美好人生</t>
+          <t>小鱼儿</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -2254,7 +2259,7 @@
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 10:19:59</t>
+          <t>2026-09-05 13:03:43</t>
         </is>
       </c>
       <c r="H37" s="0" t="inlineStr">
@@ -2264,7 +2269,7 @@
       </c>
       <c r="I37" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J37" s="0" t="inlineStr">
@@ -2285,11 +2290,11 @@
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="0">
-        <v>50074273</v>
+        <v>50080525</v>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>周利平</t>
+          <t>辞芝锦😎</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -2314,7 +2319,7 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 10:02:26</t>
+          <t>2026-09-05 13:03:29</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
@@ -2345,11 +2350,11 @@
     </row>
     <row r="39" spans="1:14">
       <c r="A39" s="0">
-        <v>50074103</v>
+        <v>50080523</v>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>赵香荣</t>
+          <t>早陈</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -2374,7 +2379,7 @@
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:58:29</t>
+          <t>2026-09-05 13:03:21</t>
         </is>
       </c>
       <c r="H39" s="0" t="inlineStr">
@@ -2405,11 +2410,11 @@
     </row>
     <row r="40" spans="1:14">
       <c r="A40" s="0">
-        <v>50074078</v>
+        <v>50080516</v>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>长风渡℡明</t>
+          <t>星星の恋人</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -2434,7 +2439,7 @@
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:49</t>
+          <t>2026-09-05 13:03:13</t>
         </is>
       </c>
       <c r="H40" s="0" t="inlineStr">
@@ -2465,11 +2470,11 @@
     </row>
     <row r="41" spans="1:14">
       <c r="A41" s="0">
-        <v>50074077</v>
+        <v>50080511</v>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>海阔天空bi</t>
+          <t>无咎</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -2494,7 +2499,7 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:47</t>
+          <t>2026-09-05 13:03:09</t>
         </is>
       </c>
       <c r="H41" s="0" t="inlineStr">
@@ -2525,11 +2530,11 @@
     </row>
     <row r="42" spans="1:14">
       <c r="A42" s="0">
-        <v>50074076</v>
+        <v>50080477</v>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>枫叶红</t>
+          <t>刘小虎</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -2554,7 +2559,7 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:47</t>
+          <t>2026-09-05 13:02:37</t>
         </is>
       </c>
       <c r="H42" s="0" t="inlineStr">
@@ -2585,11 +2590,11 @@
     </row>
     <row r="43" spans="1:14">
       <c r="A43" s="0">
-        <v>50074071</v>
+        <v>50074867</v>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>思缘</t>
+          <t>美好人生</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -2614,7 +2619,7 @@
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:35</t>
+          <t>2026-09-05 10:19:59</t>
         </is>
       </c>
       <c r="H43" s="0" t="inlineStr">
@@ -2624,7 +2629,7 @@
       </c>
       <c r="I43" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J43" s="0" t="inlineStr">
@@ -2645,11 +2650,11 @@
     </row>
     <row r="44" spans="1:14">
       <c r="A44" s="0">
-        <v>50074067</v>
+        <v>50074273</v>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>悠然</t>
+          <t>周利平</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -2674,7 +2679,7 @@
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:25</t>
+          <t>2026-09-05 10:02:26</t>
         </is>
       </c>
       <c r="H44" s="0" t="inlineStr">
@@ -2705,11 +2710,11 @@
     </row>
     <row r="45" spans="1:14">
       <c r="A45" s="0">
-        <v>50058017</v>
+        <v>50074103</v>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>索描贾师＃壹皇贰金山玉旗🇨🇳</t>
+          <t>赵香荣</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -2734,7 +2739,7 @@
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:16:49</t>
+          <t>2026-09-05 09:58:29</t>
         </is>
       </c>
       <c r="H45" s="0" t="inlineStr">
@@ -2765,11 +2770,11 @@
     </row>
     <row r="46" spans="1:14">
       <c r="A46" s="0">
-        <v>50057895</v>
+        <v>50074078</v>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>南雪</t>
+          <t>长风渡℡明</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -2794,7 +2799,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:12:32</t>
+          <t>2026-09-05 09:57:49</t>
         </is>
       </c>
       <c r="H46" s="0" t="inlineStr">
@@ -2820,21 +2825,16 @@
       <c r="L46" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N46" s="0" t="inlineStr">
-        <is>
-          <t>镇江</t>
         </is>
       </c>
     </row>
     <row r="47" spans="1:14">
       <c r="A47" s="0">
-        <v>50057857</v>
+        <v>50074077</v>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>可心</t>
+          <t>海阔天空bi</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:55</t>
+          <t>2026-09-05 09:57:47</t>
         </is>
       </c>
       <c r="H47" s="0" t="inlineStr">
@@ -2890,11 +2890,11 @@
     </row>
     <row r="48" spans="1:14">
       <c r="A48" s="0">
-        <v>50057854</v>
+        <v>50074076</v>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>张苏龙</t>
+          <t>枫叶红</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:51</t>
+          <t>2026-09-05 09:57:47</t>
         </is>
       </c>
       <c r="H48" s="0" t="inlineStr">
@@ -2950,11 +2950,11 @@
     </row>
     <row r="49" spans="1:14">
       <c r="A49" s="0">
-        <v>50057852</v>
+        <v>50074071</v>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>？</t>
+          <t>思缘</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:43</t>
+          <t>2026-09-05 09:57:35</t>
         </is>
       </c>
       <c r="H49" s="0" t="inlineStr">
@@ -3010,11 +3010,11 @@
     </row>
     <row r="50" spans="1:14">
       <c r="A50" s="0">
-        <v>50057841</v>
+        <v>50074067</v>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>向往的生活-电信号</t>
+          <t>悠然</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:09</t>
+          <t>2026-09-05 09:57:25</t>
         </is>
       </c>
       <c r="H50" s="0" t="inlineStr">
@@ -3070,11 +3070,11 @@
     </row>
     <row r="51" spans="1:14">
       <c r="A51" s="0">
-        <v>50057839</v>
+        <v>50058017</v>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>金盏花</t>
+          <t>索描贾师＃壹皇贰金山玉旗🇨🇳</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:03</t>
+          <t>2026-09-04 23:16:49</t>
         </is>
       </c>
       <c r="H51" s="0" t="inlineStr">
@@ -3130,11 +3130,11 @@
     </row>
     <row r="52" spans="1:14">
       <c r="A52" s="0">
-        <v>50032697</v>
+        <v>50057895</v>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>小米. ᩚ</t>
+          <t>南雪</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:24:13</t>
+          <t>2026-09-04 23:12:32</t>
         </is>
       </c>
       <c r="H52" s="0" t="inlineStr">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="I52" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J52" s="0" t="inlineStr">
@@ -3185,16 +3185,21 @@
       <c r="L52" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N52" s="0" t="inlineStr">
+        <is>
+          <t>镇江</t>
         </is>
       </c>
     </row>
     <row r="53" spans="1:14">
       <c r="A53" s="0">
-        <v>50032693</v>
+        <v>50057857</v>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>海岸</t>
+          <t>可心</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -3219,7 +3224,7 @@
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:24:11</t>
+          <t>2026-09-04 23:10:55</t>
         </is>
       </c>
       <c r="H53" s="0" t="inlineStr">
@@ -3229,7 +3234,7 @@
       </c>
       <c r="I53" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J53" s="0" t="inlineStr">
@@ -3250,11 +3255,11 @@
     </row>
     <row r="54" spans="1:14">
       <c r="A54" s="0">
-        <v>50032683</v>
+        <v>50057854</v>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>陆建军</t>
+          <t>张苏龙</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -3279,7 +3284,7 @@
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:23:53</t>
+          <t>2026-09-04 23:10:51</t>
         </is>
       </c>
       <c r="H54" s="0" t="inlineStr">
@@ -3289,7 +3294,7 @@
       </c>
       <c r="I54" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J54" s="0" t="inlineStr">
@@ -3310,11 +3315,11 @@
     </row>
     <row r="55" spans="1:14">
       <c r="A55" s="0">
-        <v>50015883</v>
+        <v>50057852</v>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>A00金华义乌叉车出租电15268650979</t>
+          <t>？</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -3339,7 +3344,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:18:02</t>
+          <t>2026-09-04 23:10:43</t>
         </is>
       </c>
       <c r="H55" s="0" t="inlineStr">
@@ -3349,7 +3354,7 @@
       </c>
       <c r="I55" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J55" s="0" t="inlineStr">
@@ -3370,11 +3375,11 @@
     </row>
     <row r="56" spans="1:14">
       <c r="A56" s="0">
-        <v>50015882</v>
+        <v>50057841</v>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>建程仓储中心 张川</t>
+          <t>向往的生活-电信号</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -3399,7 +3404,7 @@
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:18:02</t>
+          <t>2026-09-04 23:10:09</t>
         </is>
       </c>
       <c r="H56" s="0" t="inlineStr">
@@ -3430,11 +3435,11 @@
     </row>
     <row r="57" spans="1:14">
       <c r="A57" s="0">
-        <v>50015784</v>
+        <v>50057839</v>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>天空</t>
+          <t>金盏花</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -3459,7 +3464,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:41</t>
+          <t>2026-09-04 23:10:03</t>
         </is>
       </c>
       <c r="H57" s="0" t="inlineStr">
@@ -3490,11 +3495,11 @@
     </row>
     <row r="58" spans="1:14">
       <c r="A58" s="0">
-        <v>50015778</v>
+        <v>50032697</v>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>小龙女</t>
+          <t>小米. ᩚ</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -3519,7 +3524,7 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:21</t>
+          <t>2026-09-04 12:24:13</t>
         </is>
       </c>
       <c r="H58" s="0" t="inlineStr">
@@ -3529,7 +3534,7 @@
       </c>
       <c r="I58" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J58" s="0" t="inlineStr">
@@ -3550,11 +3555,11 @@
     </row>
     <row r="59" spans="1:14">
       <c r="A59" s="0">
-        <v>50015776</v>
+        <v>50032693</v>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>桥梁</t>
+          <t>海岸</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -3579,7 +3584,7 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:15</t>
+          <t>2026-09-04 12:24:11</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
@@ -3589,7 +3594,7 @@
       </c>
       <c r="I59" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J59" s="0" t="inlineStr">
@@ -3610,11 +3615,11 @@
     </row>
     <row r="60" spans="1:14">
       <c r="A60" s="0">
-        <v>50015775</v>
+        <v>50032683</v>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>彩云之南</t>
+          <t>陆建军</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -3639,7 +3644,7 @@
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:13</t>
+          <t>2026-09-04 12:23:53</t>
         </is>
       </c>
       <c r="H60" s="0" t="inlineStr">
@@ -3649,7 +3654,7 @@
       </c>
       <c r="I60" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J60" s="0" t="inlineStr">
@@ -3670,11 +3675,11 @@
     </row>
     <row r="61" spans="1:14">
       <c r="A61" s="0">
-        <v>50015774</v>
+        <v>50015883</v>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>楊精蓄銳༒</t>
+          <t>A00金华义乌叉车出租电15268650979</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -3699,7 +3704,7 @@
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:11</t>
+          <t>2026-09-03 23:18:02</t>
         </is>
       </c>
       <c r="H61" s="0" t="inlineStr">
@@ -3709,7 +3714,7 @@
       </c>
       <c r="I61" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J61" s="0" t="inlineStr">
@@ -3730,11 +3735,11 @@
     </row>
     <row r="62" spans="1:14">
       <c r="A62" s="0">
-        <v>50015772</v>
+        <v>50015882</v>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>不倒翁</t>
+          <t>建程仓储中心 张川</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -3759,7 +3764,7 @@
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:07</t>
+          <t>2026-09-03 23:18:02</t>
         </is>
       </c>
       <c r="H62" s="0" t="inlineStr">
@@ -3790,11 +3795,11 @@
     </row>
     <row r="63" spans="1:14">
       <c r="A63" s="0">
-        <v>50015770</v>
+        <v>50015784</v>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>一江春水</t>
+          <t>天空</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -3819,7 +3824,7 @@
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:05</t>
+          <t>2026-09-03 23:10:41</t>
         </is>
       </c>
       <c r="H63" s="0" t="inlineStr">
@@ -3850,11 +3855,11 @@
     </row>
     <row r="64" spans="1:14">
       <c r="A64" s="0">
-        <v>50015767</v>
+        <v>50015778</v>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>微笑</t>
+          <t>小龙女</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -3879,7 +3884,7 @@
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:03</t>
+          <t>2026-09-03 23:10:21</t>
         </is>
       </c>
       <c r="H64" s="0" t="inlineStr">
@@ -3910,11 +3915,11 @@
     </row>
     <row r="65" spans="1:14">
       <c r="A65" s="0">
-        <v>50015763</v>
+        <v>50015776</v>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>北斗星</t>
+          <t>桥梁</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -3939,7 +3944,7 @@
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:09:39</t>
+          <t>2026-09-03 23:10:15</t>
         </is>
       </c>
       <c r="H65" s="0" t="inlineStr">
@@ -3970,11 +3975,11 @@
     </row>
     <row r="66" spans="1:14">
       <c r="A66" s="0">
-        <v>49989442</v>
+        <v>50015775</v>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>冬梅花儿开王丽君</t>
+          <t>彩云之南</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -3999,7 +4004,7 @@
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:43</t>
+          <t>2026-09-03 23:10:13</t>
         </is>
       </c>
       <c r="H66" s="0" t="inlineStr">
@@ -4009,7 +4014,7 @@
       </c>
       <c r="I66" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J66" s="0" t="inlineStr">
@@ -4030,11 +4035,11 @@
     </row>
     <row r="67" spans="1:14">
       <c r="A67" s="0">
-        <v>49989431</v>
+        <v>50015774</v>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>风声</t>
+          <t>楊精蓄銳༒</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -4059,7 +4064,7 @@
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:25</t>
+          <t>2026-09-03 23:10:11</t>
         </is>
       </c>
       <c r="H67" s="0" t="inlineStr">
@@ -4069,7 +4074,7 @@
       </c>
       <c r="I67" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J67" s="0" t="inlineStr">
@@ -4090,11 +4095,11 @@
     </row>
     <row r="68" spans="1:14">
       <c r="A68" s="0">
-        <v>49989419</v>
+        <v>50015772</v>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>胡宾</t>
+          <t>不倒翁</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -4119,7 +4124,7 @@
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:13</t>
+          <t>2026-09-03 23:10:07</t>
         </is>
       </c>
       <c r="H68" s="0" t="inlineStr">
@@ -4129,7 +4134,7 @@
       </c>
       <c r="I68" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J68" s="0" t="inlineStr">
@@ -4150,11 +4155,11 @@
     </row>
     <row r="69" spans="1:14">
       <c r="A69" s="0">
-        <v>49989410</v>
+        <v>50015770</v>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>永远</t>
+          <t>一江春水</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -4179,7 +4184,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:03</t>
+          <t>2026-09-03 23:10:05</t>
         </is>
       </c>
       <c r="H69" s="0" t="inlineStr">
@@ -4189,7 +4194,7 @@
       </c>
       <c r="I69" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J69" s="0" t="inlineStr">
@@ -4210,11 +4215,11 @@
     </row>
     <row r="70" spans="1:14">
       <c r="A70" s="0">
-        <v>49984259</v>
+        <v>50015767</v>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>好运包张</t>
+          <t>微笑</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -4239,7 +4244,7 @@
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:55:37</t>
+          <t>2026-09-03 23:10:03</t>
         </is>
       </c>
       <c r="H70" s="0" t="inlineStr">
@@ -4249,7 +4254,7 @@
       </c>
       <c r="I70" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J70" s="0" t="inlineStr">
@@ -4270,11 +4275,11 @@
     </row>
     <row r="71" spans="1:14">
       <c r="A71" s="0">
-        <v>49984055</v>
+        <v>50015763</v>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>点点星辰</t>
+          <t>北斗星</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -4299,7 +4304,7 @@
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:49:33</t>
+          <t>2026-09-03 23:09:39</t>
         </is>
       </c>
       <c r="H71" s="0" t="inlineStr">
@@ -4330,11 +4335,11 @@
     </row>
     <row r="72" spans="1:14">
       <c r="A72" s="0">
-        <v>49983134</v>
+        <v>49989442</v>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>Zhangrruzhen张如真</t>
+          <t>冬梅花儿开王丽君</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -4359,7 +4364,7 @@
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:25:21</t>
+          <t>2026-09-03 12:23:43</t>
         </is>
       </c>
       <c r="H72" s="0" t="inlineStr">
@@ -4369,7 +4374,7 @@
       </c>
       <c r="I72" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J72" s="0" t="inlineStr">
@@ -4390,11 +4395,11 @@
     </row>
     <row r="73" spans="1:14">
       <c r="A73" s="0">
-        <v>49971209</v>
+        <v>49989431</v>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>顺丰顺水</t>
+          <t>风声</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -4419,7 +4424,7 @@
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:29:41</t>
+          <t>2026-09-03 12:23:25</t>
         </is>
       </c>
       <c r="H73" s="0" t="inlineStr">
@@ -4429,7 +4434,7 @@
       </c>
       <c r="I73" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J73" s="0" t="inlineStr">
@@ -4450,11 +4455,11 @@
     </row>
     <row r="74" spans="1:14">
       <c r="A74" s="0">
-        <v>49970732</v>
+        <v>49989419</v>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>胡宾</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -4479,7 +4484,7 @@
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:13:53</t>
+          <t>2026-09-03 12:23:13</t>
         </is>
       </c>
       <c r="H74" s="0" t="inlineStr">
@@ -4489,7 +4494,7 @@
       </c>
       <c r="I74" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J74" s="0" t="inlineStr">
@@ -4510,11 +4515,11 @@
     </row>
     <row r="75" spans="1:14">
       <c r="A75" s="0">
-        <v>49970712</v>
+        <v>49989410</v>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>月色琴弦</t>
+          <t>永远</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -4539,7 +4544,7 @@
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:13:07</t>
+          <t>2026-09-03 12:23:03</t>
         </is>
       </c>
       <c r="H75" s="0" t="inlineStr">
@@ -4549,7 +4554,7 @@
       </c>
       <c r="I75" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J75" s="0" t="inlineStr">
@@ -4570,11 +4575,11 @@
     </row>
     <row r="76" spans="1:14">
       <c r="A76" s="0">
-        <v>49970699</v>
+        <v>49984259</v>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>铜铃</t>
+          <t>好运包张</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -4599,7 +4604,7 @@
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:49</t>
+          <t>2026-09-03 09:55:37</t>
         </is>
       </c>
       <c r="H76" s="0" t="inlineStr">
@@ -4609,7 +4614,7 @@
       </c>
       <c r="I76" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J76" s="0" t="inlineStr">
@@ -4630,11 +4635,11 @@
     </row>
     <row r="77" spans="1:14">
       <c r="A77" s="0">
-        <v>49970698</v>
+        <v>49984055</v>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>东风吹</t>
+          <t>点点星辰</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -4659,7 +4664,7 @@
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:47</t>
+          <t>2026-09-03 09:49:33</t>
         </is>
       </c>
       <c r="H77" s="0" t="inlineStr">
@@ -4690,11 +4695,11 @@
     </row>
     <row r="78" spans="1:14">
       <c r="A78" s="0">
-        <v>49970683</v>
+        <v>49983134</v>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>杨永强</t>
+          <t>Zhangrruzhen张如真</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -4719,7 +4724,7 @@
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:17</t>
+          <t>2026-09-03 09:25:21</t>
         </is>
       </c>
       <c r="H78" s="0" t="inlineStr">
@@ -4729,7 +4734,7 @@
       </c>
       <c r="I78" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J78" s="0" t="inlineStr">
@@ -4750,11 +4755,11 @@
     </row>
     <row r="79" spans="1:14">
       <c r="A79" s="0">
-        <v>49970662</v>
+        <v>49971209</v>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>盈丰</t>
+          <t>顺丰顺水</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -4779,7 +4784,7 @@
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:33</t>
+          <t>2026-09-02 23:29:41</t>
         </is>
       </c>
       <c r="H79" s="0" t="inlineStr">
@@ -4810,11 +4815,11 @@
     </row>
     <row r="80" spans="1:14">
       <c r="A80" s="0">
-        <v>49970652</v>
+        <v>49970732</v>
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>YAN</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -4839,7 +4844,7 @@
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:15</t>
+          <t>2026-09-02 23:13:53</t>
         </is>
       </c>
       <c r="H80" s="0" t="inlineStr">
@@ -4870,11 +4875,11 @@
     </row>
     <row r="81" spans="1:14">
       <c r="A81" s="0">
-        <v>49970649</v>
+        <v>49970712</v>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>彩虹（宋荷娣）</t>
+          <t>月色琴弦</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -4899,7 +4904,7 @@
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:11</t>
+          <t>2026-09-02 23:13:07</t>
         </is>
       </c>
       <c r="H81" s="0" t="inlineStr">
@@ -4930,11 +4935,11 @@
     </row>
     <row r="82" spans="1:14">
       <c r="A82" s="0">
-        <v>49970648</v>
+        <v>49970699</v>
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>天知心</t>
+          <t>铜铃</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -4959,7 +4964,7 @@
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:08</t>
+          <t>2026-09-02 23:12:49</t>
         </is>
       </c>
       <c r="H82" s="0" t="inlineStr">
@@ -4990,11 +4995,11 @@
     </row>
     <row r="83" spans="1:14">
       <c r="A83" s="0">
-        <v>49970643</v>
+        <v>49970698</v>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>好运来</t>
+          <t>东风吹</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -5019,7 +5024,7 @@
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:10:55</t>
+          <t>2026-09-02 23:12:47</t>
         </is>
       </c>
       <c r="H83" s="0" t="inlineStr">
@@ -5050,11 +5055,11 @@
     </row>
     <row r="84" spans="1:14">
       <c r="A84" s="0">
-        <v>49937566</v>
+        <v>49970683</v>
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>简单sincerity</t>
+          <t>杨永强</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -5079,7 +5084,7 @@
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 10:10:33</t>
+          <t>2026-09-02 23:12:17</t>
         </is>
       </c>
       <c r="H84" s="0" t="inlineStr">
@@ -5110,11 +5115,11 @@
     </row>
     <row r="85" spans="1:14">
       <c r="A85" s="0">
-        <v>49937187</v>
+        <v>49970662</v>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>莲子</t>
+          <t>盈丰</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -5139,7 +5144,7 @@
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:58:56</t>
+          <t>2026-09-02 23:11:33</t>
         </is>
       </c>
       <c r="H85" s="0" t="inlineStr">
@@ -5149,7 +5154,7 @@
       </c>
       <c r="I85" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J85" s="0" t="inlineStr">
@@ -5170,11 +5175,11 @@
     </row>
     <row r="86" spans="1:14">
       <c r="A86" s="0">
-        <v>49937101</v>
+        <v>49970652</v>
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>蓉儿</t>
+          <t>YAN</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -5199,7 +5204,7 @@
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:56:16</t>
+          <t>2026-09-02 23:11:15</t>
         </is>
       </c>
       <c r="H86" s="0" t="inlineStr">
@@ -5230,11 +5235,11 @@
     </row>
     <row r="87" spans="1:14">
       <c r="A87" s="0">
-        <v>49937098</v>
+        <v>49970649</v>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>瀚林2368</t>
+          <t>彩虹（宋荷娣）</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -5259,7 +5264,7 @@
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:56:15</t>
+          <t>2026-09-02 23:11:11</t>
         </is>
       </c>
       <c r="H87" s="0" t="inlineStr">
@@ -5290,11 +5295,11 @@
     </row>
     <row r="88" spans="1:14">
       <c r="A88" s="0">
-        <v>49937081</v>
+        <v>49970648</v>
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>🔱 花中之美</t>
+          <t>天知心</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -5319,7 +5324,7 @@
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:47</t>
+          <t>2026-09-02 23:11:08</t>
         </is>
       </c>
       <c r="H88" s="0" t="inlineStr">
@@ -5350,11 +5355,11 @@
     </row>
     <row r="89" spans="1:14">
       <c r="A89" s="0">
-        <v>49937066</v>
+        <v>49970643</v>
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>雨情</t>
+          <t>好运来</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -5379,7 +5384,7 @@
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:27</t>
+          <t>2026-09-02 23:10:55</t>
         </is>
       </c>
       <c r="H89" s="0" t="inlineStr">
@@ -5410,11 +5415,11 @@
     </row>
     <row r="90" spans="1:14">
       <c r="A90" s="0">
-        <v>49937061</v>
+        <v>49937566</v>
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>Sunny 🎈瑶</t>
+          <t>简单sincerity</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -5439,7 +5444,7 @@
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:23</t>
+          <t>2026-09-02 10:10:33</t>
         </is>
       </c>
       <c r="H90" s="0" t="inlineStr">
@@ -5470,11 +5475,11 @@
     </row>
     <row r="91" spans="1:14">
       <c r="A91" s="0">
-        <v>49887876</v>
+        <v>49937187</v>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>鱼靖儿</t>
+          <t>莲子</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -5499,7 +5504,7 @@
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:23:11</t>
+          <t>2026-09-02 09:58:56</t>
         </is>
       </c>
       <c r="H91" s="0" t="inlineStr">
@@ -5530,11 +5535,11 @@
     </row>
     <row r="92" spans="1:14">
       <c r="A92" s="0">
-        <v>49887478</v>
+        <v>49937101</v>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t>风调雨顺</t>
+          <t>蓉儿</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -5559,7 +5564,7 @@
       </c>
       <c r="G92" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:10:17</t>
+          <t>2026-09-02 09:56:16</t>
         </is>
       </c>
       <c r="H92" s="0" t="inlineStr">
@@ -5590,11 +5595,11 @@
     </row>
     <row r="93" spans="1:14">
       <c r="A93" s="0">
-        <v>49887447</v>
+        <v>49937098</v>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t>中国艺人</t>
+          <t>瀚林2368</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -5619,7 +5624,7 @@
       </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:44</t>
+          <t>2026-09-02 09:56:15</t>
         </is>
       </c>
       <c r="H93" s="0" t="inlineStr">
@@ -5650,11 +5655,11 @@
     </row>
     <row r="94" spans="1:14">
       <c r="A94" s="0">
-        <v>49887439</v>
+        <v>49937081</v>
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t>黄晓玲</t>
+          <t>🔱 花中之美</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
@@ -5679,7 +5684,7 @@
       </c>
       <c r="G94" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:17</t>
+          <t>2026-09-02 09:55:47</t>
         </is>
       </c>
       <c r="H94" s="0" t="inlineStr">
@@ -5710,11 +5715,11 @@
     </row>
     <row r="95" spans="1:14">
       <c r="A95" s="0">
-        <v>49887437</v>
+        <v>49937066</v>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>随缘</t>
+          <t>雨情</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">
@@ -5739,7 +5744,7 @@
       </c>
       <c r="G95" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:07</t>
+          <t>2026-09-02 09:55:27</t>
         </is>
       </c>
       <c r="H95" s="0" t="inlineStr">
@@ -5770,11 +5775,11 @@
     </row>
     <row r="96" spans="1:14">
       <c r="A96" s="0">
-        <v>49887416</v>
+        <v>49937061</v>
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t>刘秋红</t>
+          <t>Sunny 🎈瑶</t>
         </is>
       </c>
       <c r="C96" s="0" t="inlineStr">
@@ -5799,7 +5804,7 @@
       </c>
       <c r="G96" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:31</t>
+          <t>2026-09-02 09:55:23</t>
         </is>
       </c>
       <c r="H96" s="0" t="inlineStr">
@@ -5830,11 +5835,11 @@
     </row>
     <row r="97" spans="1:14">
       <c r="A97" s="0">
-        <v>49887403</v>
+        <v>49887876</v>
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>Mr.</t>
+          <t>鱼靖儿</t>
         </is>
       </c>
       <c r="C97" s="0" t="inlineStr">
@@ -5859,7 +5864,7 @@
       </c>
       <c r="G97" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:05</t>
+          <t>2026-08-31 23:23:11</t>
         </is>
       </c>
       <c r="H97" s="0" t="inlineStr">
@@ -5869,7 +5874,7 @@
       </c>
       <c r="I97" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J97" s="0" t="inlineStr">
@@ -5890,11 +5895,11 @@
     </row>
     <row r="98" spans="1:14">
       <c r="A98" s="0">
-        <v>49887401</v>
+        <v>49887478</v>
       </c>
       <c r="B98" s="0" t="inlineStr">
         <is>
-          <t>万事如意</t>
+          <t>风调雨顺</t>
         </is>
       </c>
       <c r="C98" s="0" t="inlineStr">
@@ -5919,7 +5924,7 @@
       </c>
       <c r="G98" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:03</t>
+          <t>2026-08-31 23:10:17</t>
         </is>
       </c>
       <c r="H98" s="0" t="inlineStr">
@@ -5950,11 +5955,11 @@
     </row>
     <row r="99" spans="1:14">
       <c r="A99" s="0">
-        <v>49887400</v>
+        <v>49887447</v>
       </c>
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t>💋诺墨</t>
+          <t>中国艺人</t>
         </is>
       </c>
       <c r="C99" s="0" t="inlineStr">
@@ -5979,7 +5984,7 @@
       </c>
       <c r="G99" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:01</t>
+          <t>2026-08-31 23:08:44</t>
         </is>
       </c>
       <c r="H99" s="0" t="inlineStr">
@@ -6010,11 +6015,11 @@
     </row>
     <row r="100" spans="1:14">
       <c r="A100" s="0">
-        <v>49887399</v>
+        <v>49887439</v>
       </c>
       <c r="B100" s="0" t="inlineStr">
         <is>
-          <t>听风</t>
+          <t>黄晓玲</t>
         </is>
       </c>
       <c r="C100" s="0" t="inlineStr">
@@ -6039,7 +6044,7 @@
       </c>
       <c r="G100" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:06:59</t>
+          <t>2026-08-31 23:08:17</t>
         </is>
       </c>
       <c r="H100" s="0" t="inlineStr">
@@ -6070,11 +6075,11 @@
     </row>
     <row r="101" spans="1:14">
       <c r="A101" s="0">
-        <v>49845584</v>
+        <v>49887437</v>
       </c>
       <c r="B101" s="0" t="inlineStr">
         <is>
-          <t>彭汉平13024282926</t>
+          <t>随缘</t>
         </is>
       </c>
       <c r="C101" s="0" t="inlineStr">
@@ -6099,7 +6104,7 @@
       </c>
       <c r="G101" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:18:55</t>
+          <t>2026-08-31 23:08:07</t>
         </is>
       </c>
       <c r="H101" s="0" t="inlineStr">
@@ -6130,11 +6135,11 @@
     </row>
     <row r="102" spans="1:14">
       <c r="A102" s="0">
-        <v>49845487</v>
+        <v>49887416</v>
       </c>
       <c r="B102" s="0" t="inlineStr">
         <is>
-          <t>Z国华</t>
+          <t>刘秋红</t>
         </is>
       </c>
       <c r="C102" s="0" t="inlineStr">
@@ -6159,7 +6164,7 @@
       </c>
       <c r="G102" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:15:49</t>
+          <t>2026-08-31 23:07:31</t>
         </is>
       </c>
       <c r="H102" s="0" t="inlineStr">
@@ -6169,7 +6174,7 @@
       </c>
       <c r="I102" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J102" s="0" t="inlineStr">
@@ -6190,11 +6195,11 @@
     </row>
     <row r="103" spans="1:14">
       <c r="A103" s="0">
-        <v>49845407</v>
+        <v>49887403</v>
       </c>
       <c r="B103" s="0" t="inlineStr">
         <is>
-          <t>月亮🌛</t>
+          <t>Mr.</t>
         </is>
       </c>
       <c r="C103" s="0" t="inlineStr">
@@ -6219,7 +6224,7 @@
       </c>
       <c r="G103" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:12:33</t>
+          <t>2026-08-31 23:07:05</t>
         </is>
       </c>
       <c r="H103" s="0" t="inlineStr">
@@ -6250,11 +6255,11 @@
     </row>
     <row r="104" spans="1:14">
       <c r="A104" s="0">
-        <v>49845398</v>
+        <v>49887401</v>
       </c>
       <c r="B104" s="0" t="inlineStr">
         <is>
-          <t>老树</t>
+          <t>万事如意</t>
         </is>
       </c>
       <c r="C104" s="0" t="inlineStr">
@@ -6279,7 +6284,7 @@
       </c>
       <c r="G104" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:12:03</t>
+          <t>2026-08-31 23:07:03</t>
         </is>
       </c>
       <c r="H104" s="0" t="inlineStr">
@@ -6310,11 +6315,11 @@
     </row>
     <row r="105" spans="1:14">
       <c r="A105" s="0">
-        <v>49845391</v>
+        <v>49887400</v>
       </c>
       <c r="B105" s="0" t="inlineStr">
         <is>
-          <t>八哥</t>
+          <t>💋诺墨</t>
         </is>
       </c>
       <c r="C105" s="0" t="inlineStr">
@@ -6339,7 +6344,7 @@
       </c>
       <c r="G105" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:45</t>
+          <t>2026-08-31 23:07:01</t>
         </is>
       </c>
       <c r="H105" s="0" t="inlineStr">
@@ -6370,11 +6375,11 @@
     </row>
     <row r="106" spans="1:14">
       <c r="A106" s="0">
-        <v>49845380</v>
+        <v>49887399</v>
       </c>
       <c r="B106" s="0" t="inlineStr">
         <is>
-          <t>铲车主出租15352562068</t>
+          <t>听风</t>
         </is>
       </c>
       <c r="C106" s="0" t="inlineStr">
@@ -6399,7 +6404,7 @@
       </c>
       <c r="G106" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:29</t>
+          <t>2026-08-31 23:06:59</t>
         </is>
       </c>
       <c r="H106" s="0" t="inlineStr">
@@ -6430,11 +6435,11 @@
     </row>
     <row r="107" spans="1:14">
       <c r="A107" s="0">
-        <v>49845376</v>
+        <v>49845584</v>
       </c>
       <c r="B107" s="0" t="inlineStr">
         <is>
-          <t>刘萍</t>
+          <t>彭汉平13024282926</t>
         </is>
       </c>
       <c r="C107" s="0" t="inlineStr">
@@ -6459,7 +6464,7 @@
       </c>
       <c r="G107" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:15</t>
+          <t>2026-08-30 23:18:55</t>
         </is>
       </c>
       <c r="H107" s="0" t="inlineStr">
@@ -6490,11 +6495,11 @@
     </row>
     <row r="108" spans="1:14">
       <c r="A108" s="0">
-        <v>49845374</v>
+        <v>49845487</v>
       </c>
       <c r="B108" s="0" t="inlineStr">
         <is>
-          <t>空谷幽兰</t>
+          <t>Z国华</t>
         </is>
       </c>
       <c r="C108" s="0" t="inlineStr">
@@ -6519,7 +6524,7 @@
       </c>
       <c r="G108" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:07</t>
+          <t>2026-08-30 23:15:49</t>
         </is>
       </c>
       <c r="H108" s="0" t="inlineStr">
@@ -6529,7 +6534,7 @@
       </c>
       <c r="I108" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J108" s="0" t="inlineStr">
@@ -6550,11 +6555,11 @@
     </row>
     <row r="109" spans="1:14">
       <c r="A109" s="0">
-        <v>49845373</v>
+        <v>49845407</v>
       </c>
       <c r="B109" s="0" t="inlineStr">
         <is>
-          <t>泽浩羊</t>
+          <t>月亮🌛</t>
         </is>
       </c>
       <c r="C109" s="0" t="inlineStr">
@@ -6579,7 +6584,7 @@
       </c>
       <c r="G109" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:05</t>
+          <t>2026-08-30 23:12:33</t>
         </is>
       </c>
       <c r="H109" s="0" t="inlineStr">
@@ -6610,11 +6615,11 @@
     </row>
     <row r="110" spans="1:14">
       <c r="A110" s="0">
-        <v>49845367</v>
+        <v>49845398</v>
       </c>
       <c r="B110" s="0" t="inlineStr">
         <is>
-          <t>峰回路转</t>
+          <t>老树</t>
         </is>
       </c>
       <c r="C110" s="0" t="inlineStr">
@@ -6639,7 +6644,7 @@
       </c>
       <c r="G110" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:55</t>
+          <t>2026-08-30 23:12:03</t>
         </is>
       </c>
       <c r="H110" s="0" t="inlineStr">
@@ -6670,11 +6675,11 @@
     </row>
     <row r="111" spans="1:14">
       <c r="A111" s="0">
-        <v>49845366</v>
+        <v>49845391</v>
       </c>
       <c r="B111" s="0" t="inlineStr">
         <is>
-          <t>超儿</t>
+          <t>八哥</t>
         </is>
       </c>
       <c r="C111" s="0" t="inlineStr">
@@ -6699,7 +6704,7 @@
       </c>
       <c r="G111" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:51</t>
+          <t>2026-08-30 23:11:45</t>
         </is>
       </c>
       <c r="H111" s="0" t="inlineStr">
@@ -6730,11 +6735,11 @@
     </row>
     <row r="112" spans="1:14">
       <c r="A112" s="0">
-        <v>49845365</v>
+        <v>49845380</v>
       </c>
       <c r="B112" s="0" t="inlineStr">
         <is>
-          <t>传</t>
+          <t>铲车主出租15352562068</t>
         </is>
       </c>
       <c r="C112" s="0" t="inlineStr">
@@ -6759,7 +6764,7 @@
       </c>
       <c r="G112" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:49</t>
+          <t>2026-08-30 23:11:29</t>
         </is>
       </c>
       <c r="H112" s="0" t="inlineStr">
@@ -6790,11 +6795,11 @@
     </row>
     <row r="113" spans="1:14">
       <c r="A113" s="0">
-        <v>49845360</v>
+        <v>49845376</v>
       </c>
       <c r="B113" s="0" t="inlineStr">
         <is>
-          <t>悟歌</t>
+          <t>刘萍</t>
         </is>
       </c>
       <c r="C113" s="0" t="inlineStr">
@@ -6819,7 +6824,7 @@
       </c>
       <c r="G113" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:43</t>
+          <t>2026-08-30 23:11:15</t>
         </is>
       </c>
       <c r="H113" s="0" t="inlineStr">
@@ -6850,11 +6855,11 @@
     </row>
     <row r="114" spans="1:14">
       <c r="A114" s="0">
-        <v>49845342</v>
+        <v>49845374</v>
       </c>
       <c r="B114" s="0" t="inlineStr">
         <is>
-          <t>丽丽</t>
+          <t>空谷幽兰</t>
         </is>
       </c>
       <c r="C114" s="0" t="inlineStr">
@@ -6879,7 +6884,7 @@
       </c>
       <c r="G114" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:15</t>
+          <t>2026-08-30 23:11:07</t>
         </is>
       </c>
       <c r="H114" s="0" t="inlineStr">
@@ -6910,11 +6915,11 @@
     </row>
     <row r="115" spans="1:14">
       <c r="A115" s="0">
-        <v>49826011</v>
+        <v>49845373</v>
       </c>
       <c r="B115" s="0" t="inlineStr">
         <is>
-          <t>王前卫</t>
+          <t>泽浩羊</t>
         </is>
       </c>
       <c r="C115" s="0" t="inlineStr">
@@ -6939,7 +6944,7 @@
       </c>
       <c r="G115" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:57:27</t>
+          <t>2026-08-30 23:11:05</t>
         </is>
       </c>
       <c r="H115" s="0" t="inlineStr">
@@ -6970,11 +6975,11 @@
     </row>
     <row r="116" spans="1:14">
       <c r="A116" s="0">
-        <v>49825720</v>
+        <v>49845367</v>
       </c>
       <c r="B116" s="0" t="inlineStr">
         <is>
-          <t>老A</t>
+          <t>峰回路转</t>
         </is>
       </c>
       <c r="C116" s="0" t="inlineStr">
@@ -6999,7 +7004,7 @@
       </c>
       <c r="G116" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:46:02</t>
+          <t>2026-08-30 23:10:55</t>
         </is>
       </c>
       <c r="H116" s="0" t="inlineStr">
@@ -7030,11 +7035,11 @@
     </row>
     <row r="117" spans="1:14">
       <c r="A117" s="0">
-        <v>49825676</v>
+        <v>49845366</v>
       </c>
       <c r="B117" s="0" t="inlineStr">
         <is>
-          <t>蓝天</t>
+          <t>超儿</t>
         </is>
       </c>
       <c r="C117" s="0" t="inlineStr">
@@ -7059,7 +7064,7 @@
       </c>
       <c r="G117" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:44:05</t>
+          <t>2026-08-30 23:10:51</t>
         </is>
       </c>
       <c r="H117" s="0" t="inlineStr">
@@ -7090,11 +7095,11 @@
     </row>
     <row r="118" spans="1:14">
       <c r="A118" s="0">
-        <v>49825650</v>
+        <v>49845365</v>
       </c>
       <c r="B118" s="0" t="inlineStr">
         <is>
-          <t>爱芳</t>
+          <t>传</t>
         </is>
       </c>
       <c r="C118" s="0" t="inlineStr">
@@ -7119,7 +7124,7 @@
       </c>
       <c r="G118" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:43:11</t>
+          <t>2026-08-30 23:10:49</t>
         </is>
       </c>
       <c r="H118" s="0" t="inlineStr">
@@ -7150,11 +7155,11 @@
     </row>
     <row r="119" spans="1:14">
       <c r="A119" s="0">
-        <v>49825642</v>
+        <v>49845360</v>
       </c>
       <c r="B119" s="0" t="inlineStr">
         <is>
-          <t>银杏树</t>
+          <t>悟歌</t>
         </is>
       </c>
       <c r="C119" s="0" t="inlineStr">
@@ -7179,7 +7184,7 @@
       </c>
       <c r="G119" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:55</t>
+          <t>2026-08-30 23:10:43</t>
         </is>
       </c>
       <c r="H119" s="0" t="inlineStr">
@@ -7210,11 +7215,11 @@
     </row>
     <row r="120" spans="1:14">
       <c r="A120" s="0">
-        <v>49825640</v>
+        <v>49845342</v>
       </c>
       <c r="B120" s="0" t="inlineStr">
         <is>
-          <t>遵命有福（杨凤）</t>
+          <t>丽丽</t>
         </is>
       </c>
       <c r="C120" s="0" t="inlineStr">
@@ -7239,7 +7244,7 @@
       </c>
       <c r="G120" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:49</t>
+          <t>2026-08-30 23:10:15</t>
         </is>
       </c>
       <c r="H120" s="0" t="inlineStr">
@@ -7270,11 +7275,11 @@
     </row>
     <row r="121" spans="1:14">
       <c r="A121" s="0">
-        <v>49825639</v>
+        <v>49826011</v>
       </c>
       <c r="B121" s="0" t="inlineStr">
         <is>
-          <t>申华</t>
+          <t>王前卫</t>
         </is>
       </c>
       <c r="C121" s="0" t="inlineStr">
@@ -7299,7 +7304,7 @@
       </c>
       <c r="G121" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:49</t>
+          <t>2026-08-30 12:57:27</t>
         </is>
       </c>
       <c r="H121" s="0" t="inlineStr">
@@ -7330,11 +7335,11 @@
     </row>
     <row r="122" spans="1:14">
       <c r="A122" s="0">
-        <v>49825637</v>
+        <v>49825720</v>
       </c>
       <c r="B122" s="0" t="inlineStr">
         <is>
-          <t>陈月焓</t>
+          <t>老A</t>
         </is>
       </c>
       <c r="C122" s="0" t="inlineStr">
@@ -7359,7 +7364,7 @@
       </c>
       <c r="G122" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:47</t>
+          <t>2026-08-30 12:46:02</t>
         </is>
       </c>
       <c r="H122" s="0" t="inlineStr">
@@ -7390,11 +7395,11 @@
     </row>
     <row r="123" spans="1:14">
       <c r="A123" s="0">
-        <v>49825635</v>
+        <v>49825676</v>
       </c>
       <c r="B123" s="0" t="inlineStr">
         <is>
-          <t>小镇生活&amp;&amp;杜震</t>
+          <t>蓝天</t>
         </is>
       </c>
       <c r="C123" s="0" t="inlineStr">
@@ -7419,7 +7424,7 @@
       </c>
       <c r="G123" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:43</t>
+          <t>2026-08-30 12:44:05</t>
         </is>
       </c>
       <c r="H123" s="0" t="inlineStr">
@@ -7450,11 +7455,11 @@
     </row>
     <row r="124" spans="1:14">
       <c r="A124" s="0">
-        <v>49825628</v>
+        <v>49825650</v>
       </c>
       <c r="B124" s="0" t="inlineStr">
         <is>
-          <t>Taᴗaoᥫᩣ</t>
+          <t>爱芳</t>
         </is>
       </c>
       <c r="C124" s="0" t="inlineStr">
@@ -7479,7 +7484,7 @@
       </c>
       <c r="G124" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:35</t>
+          <t>2026-08-30 12:43:11</t>
         </is>
       </c>
       <c r="H124" s="0" t="inlineStr">
@@ -7510,11 +7515,11 @@
     </row>
     <row r="125" spans="1:14">
       <c r="A125" s="0">
-        <v>49782066</v>
+        <v>49825642</v>
       </c>
       <c r="B125" s="0" t="inlineStr">
         <is>
-          <t>前程似锦</t>
+          <t>银杏树</t>
         </is>
       </c>
       <c r="C125" s="0" t="inlineStr">
@@ -7539,7 +7544,7 @@
       </c>
       <c r="G125" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 09:07:29</t>
+          <t>2026-08-30 12:42:55</t>
         </is>
       </c>
       <c r="H125" s="0" t="inlineStr">
@@ -7549,7 +7554,7 @@
       </c>
       <c r="I125" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J125" s="0" t="inlineStr">
@@ -7570,11 +7575,11 @@
     </row>
     <row r="126" spans="1:14">
       <c r="A126" s="0">
-        <v>49771027</v>
+        <v>49825640</v>
       </c>
       <c r="B126" s="0" t="inlineStr">
         <is>
-          <t>非比</t>
+          <t>遵命有福（杨凤）</t>
         </is>
       </c>
       <c r="C126" s="0" t="inlineStr">
@@ -7599,7 +7604,7 @@
       </c>
       <c r="G126" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 23:30:09</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H126" s="0" t="inlineStr">
@@ -7609,7 +7614,7 @@
       </c>
       <c r="I126" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J126" s="0" t="inlineStr">
@@ -7630,11 +7635,11 @@
     </row>
     <row r="127" spans="1:14">
       <c r="A127" s="0">
-        <v>49673360</v>
+        <v>49825639</v>
       </c>
       <c r="B127" s="0" t="inlineStr">
         <is>
-          <t>德行天下</t>
+          <t>申华</t>
         </is>
       </c>
       <c r="C127" s="0" t="inlineStr">
@@ -7659,7 +7664,7 @@
       </c>
       <c r="G127" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:19:03</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H127" s="0" t="inlineStr">
@@ -7669,7 +7674,7 @@
       </c>
       <c r="I127" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J127" s="0" t="inlineStr">
@@ -7690,11 +7695,11 @@
     </row>
     <row r="128" spans="1:14">
       <c r="A128" s="0">
-        <v>49673352</v>
+        <v>49825637</v>
       </c>
       <c r="B128" s="0" t="inlineStr">
         <is>
-          <t>余盛将至2026</t>
+          <t>陈月焓</t>
         </is>
       </c>
       <c r="C128" s="0" t="inlineStr">
@@ -7719,7 +7724,7 @@
       </c>
       <c r="G128" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:49</t>
+          <t>2026-08-30 12:42:47</t>
         </is>
       </c>
       <c r="H128" s="0" t="inlineStr">
@@ -7729,7 +7734,7 @@
       </c>
       <c r="I128" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J128" s="0" t="inlineStr">
@@ -7750,11 +7755,11 @@
     </row>
     <row r="129" spans="1:14">
       <c r="A129" s="0">
-        <v>49673350</v>
+        <v>49825635</v>
       </c>
       <c r="B129" s="0" t="inlineStr">
         <is>
-          <t>山居客</t>
+          <t>小镇生活&amp;&amp;杜震</t>
         </is>
       </c>
       <c r="C129" s="0" t="inlineStr">
@@ -7779,7 +7784,7 @@
       </c>
       <c r="G129" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:47</t>
+          <t>2026-08-30 12:42:43</t>
         </is>
       </c>
       <c r="H129" s="0" t="inlineStr">
@@ -7789,7 +7794,7 @@
       </c>
       <c r="I129" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J129" s="0" t="inlineStr">
@@ -7810,11 +7815,11 @@
     </row>
     <row r="130" spans="1:14">
       <c r="A130" s="0">
-        <v>49673349</v>
+        <v>49825628</v>
       </c>
       <c r="B130" s="0" t="inlineStr">
         <is>
-          <t>白云</t>
+          <t>Taᴗaoᥫᩣ</t>
         </is>
       </c>
       <c r="C130" s="0" t="inlineStr">
@@ -7839,7 +7844,7 @@
       </c>
       <c r="G130" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:45</t>
+          <t>2026-08-30 12:42:35</t>
         </is>
       </c>
       <c r="H130" s="0" t="inlineStr">
@@ -7849,7 +7854,7 @@
       </c>
       <c r="I130" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J130" s="0" t="inlineStr">
@@ -7870,11 +7875,11 @@
     </row>
     <row r="131" spans="1:14">
       <c r="A131" s="0">
-        <v>49646935</v>
+        <v>49782066</v>
       </c>
       <c r="B131" s="0" t="inlineStr">
         <is>
-          <t>马跃荣</t>
+          <t>前程似锦</t>
         </is>
       </c>
       <c r="C131" s="0" t="inlineStr">
@@ -7899,7 +7904,7 @@
       </c>
       <c r="G131" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:59</t>
+          <t>2026-08-29 09:07:29</t>
         </is>
       </c>
       <c r="H131" s="0" t="inlineStr">
@@ -7909,7 +7914,7 @@
       </c>
       <c r="I131" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J131" s="0" t="inlineStr">
@@ -7930,11 +7935,11 @@
     </row>
     <row r="132" spans="1:14">
       <c r="A132" s="0">
-        <v>49646933</v>
+        <v>49771027</v>
       </c>
       <c r="B132" s="0" t="inlineStr">
         <is>
-          <t>@吴</t>
+          <t>非比</t>
         </is>
       </c>
       <c r="C132" s="0" t="inlineStr">
@@ -7959,7 +7964,7 @@
       </c>
       <c r="G132" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:56</t>
+          <t>2026-08-28 23:30:09</t>
         </is>
       </c>
       <c r="H132" s="0" t="inlineStr">
@@ -7969,7 +7974,7 @@
       </c>
       <c r="I132" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J132" s="0" t="inlineStr">
@@ -7990,11 +7995,11 @@
     </row>
     <row r="133" spans="1:14">
       <c r="A133" s="0">
-        <v>49646901</v>
+        <v>49673360</v>
       </c>
       <c r="B133" s="0" t="inlineStr">
         <is>
-          <t>龙安：富华／</t>
+          <t>德行天下</t>
         </is>
       </c>
       <c r="C133" s="0" t="inlineStr">
@@ -8019,7 +8024,7 @@
       </c>
       <c r="G133" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:14:28</t>
+          <t>2026-08-26 12:19:03</t>
         </is>
       </c>
       <c r="H133" s="0" t="inlineStr">
@@ -8050,11 +8055,11 @@
     </row>
     <row r="134" spans="1:14">
       <c r="A134" s="0">
-        <v>49646876</v>
+        <v>49673352</v>
       </c>
       <c r="B134" s="0" t="inlineStr">
         <is>
-          <t>冬日暖阳🌻</t>
+          <t>余盛将至2026</t>
         </is>
       </c>
       <c r="C134" s="0" t="inlineStr">
@@ -8079,7 +8084,7 @@
       </c>
       <c r="G134" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:37</t>
+          <t>2026-08-26 12:18:49</t>
         </is>
       </c>
       <c r="H134" s="0" t="inlineStr">
@@ -8110,11 +8115,11 @@
     </row>
     <row r="135" spans="1:14">
       <c r="A135" s="0">
-        <v>49646867</v>
+        <v>49673350</v>
       </c>
       <c r="B135" s="0" t="inlineStr">
         <is>
-          <t>寒雨</t>
+          <t>山居客</t>
         </is>
       </c>
       <c r="C135" s="0" t="inlineStr">
@@ -8139,7 +8144,7 @@
       </c>
       <c r="G135" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:15</t>
+          <t>2026-08-26 12:18:47</t>
         </is>
       </c>
       <c r="H135" s="0" t="inlineStr">
@@ -8170,11 +8175,11 @@
     </row>
     <row r="136" spans="1:14">
       <c r="A136" s="0">
-        <v>49636232</v>
+        <v>49673349</v>
       </c>
       <c r="B136" s="0" t="inlineStr">
         <is>
-          <t>平安</t>
+          <t>白云</t>
         </is>
       </c>
       <c r="C136" s="0" t="inlineStr">
@@ -8199,7 +8204,7 @@
       </c>
       <c r="G136" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:20:15</t>
+          <t>2026-08-26 12:18:45</t>
         </is>
       </c>
       <c r="H136" s="0" t="inlineStr">
@@ -8209,7 +8214,7 @@
       </c>
       <c r="I136" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J136" s="0" t="inlineStr">
@@ -8230,11 +8235,11 @@
     </row>
     <row r="137" spans="1:14">
       <c r="A137" s="0">
-        <v>49636184</v>
+        <v>49646935</v>
       </c>
       <c r="B137" s="0" t="inlineStr">
         <is>
-          <t>古道西风</t>
+          <t>马跃荣</t>
         </is>
       </c>
       <c r="C137" s="0" t="inlineStr">
@@ -8259,7 +8264,7 @@
       </c>
       <c r="G137" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:55</t>
+          <t>2026-08-25 18:15:59</t>
         </is>
       </c>
       <c r="H137" s="0" t="inlineStr">
@@ -8269,7 +8274,7 @@
       </c>
       <c r="I137" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J137" s="0" t="inlineStr">
@@ -8290,11 +8295,11 @@
     </row>
     <row r="138" spans="1:14">
       <c r="A138" s="0">
-        <v>49636170</v>
+        <v>49646933</v>
       </c>
       <c r="B138" s="0" t="inlineStr">
         <is>
-          <t>周海龙</t>
+          <t>@吴</t>
         </is>
       </c>
       <c r="C138" s="0" t="inlineStr">
@@ -8319,7 +8324,7 @@
       </c>
       <c r="G138" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:33</t>
+          <t>2026-08-25 18:15:56</t>
         </is>
       </c>
       <c r="H138" s="0" t="inlineStr">
@@ -8329,7 +8334,7 @@
       </c>
       <c r="I138" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J138" s="0" t="inlineStr">
@@ -8350,11 +8355,11 @@
     </row>
     <row r="139" spans="1:14">
       <c r="A139" s="0">
-        <v>49636157</v>
+        <v>49646901</v>
       </c>
       <c r="B139" s="0" t="inlineStr">
         <is>
-          <t>锦妍</t>
+          <t>龙安：富华／</t>
         </is>
       </c>
       <c r="C139" s="0" t="inlineStr">
@@ -8379,7 +8384,7 @@
       </c>
       <c r="G139" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:07</t>
+          <t>2026-08-25 18:14:28</t>
         </is>
       </c>
       <c r="H139" s="0" t="inlineStr">
@@ -8389,7 +8394,7 @@
       </c>
       <c r="I139" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J139" s="0" t="inlineStr">
@@ -8410,11 +8415,11 @@
     </row>
     <row r="140" spans="1:14">
       <c r="A140" s="0">
-        <v>49593974</v>
+        <v>49646876</v>
       </c>
       <c r="B140" s="0" t="inlineStr">
         <is>
-          <t>兰兰</t>
+          <t>冬日暖阳🌻</t>
         </is>
       </c>
       <c r="C140" s="0" t="inlineStr">
@@ -8439,7 +8444,7 @@
       </c>
       <c r="G140" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:59:53</t>
+          <t>2026-08-25 18:13:37</t>
         </is>
       </c>
       <c r="H140" s="0" t="inlineStr">
@@ -8449,7 +8454,7 @@
       </c>
       <c r="I140" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J140" s="0" t="inlineStr">
@@ -8470,11 +8475,11 @@
     </row>
     <row r="141" spans="1:14">
       <c r="A141" s="0">
-        <v>49593671</v>
+        <v>49646867</v>
       </c>
       <c r="B141" s="0" t="inlineStr">
         <is>
-          <t>准备1号</t>
+          <t>寒雨</t>
         </is>
       </c>
       <c r="C141" s="0" t="inlineStr">
@@ -8499,7 +8504,7 @@
       </c>
       <c r="G141" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:49:27</t>
+          <t>2026-08-25 18:13:15</t>
         </is>
       </c>
       <c r="H141" s="0" t="inlineStr">
@@ -8509,7 +8514,7 @@
       </c>
       <c r="I141" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J141" s="0" t="inlineStr">
@@ -8530,11 +8535,11 @@
     </row>
     <row r="142" spans="1:14">
       <c r="A142" s="0">
-        <v>49535916</v>
+        <v>49636232</v>
       </c>
       <c r="B142" s="0" t="inlineStr">
         <is>
-          <t>真诚</t>
+          <t>平安</t>
         </is>
       </c>
       <c r="C142" s="0" t="inlineStr">
@@ -8559,7 +8564,7 @@
       </c>
       <c r="G142" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:46:23</t>
+          <t>2026-08-25 13:20:15</t>
         </is>
       </c>
       <c r="H142" s="0" t="inlineStr">
@@ -8590,11 +8595,11 @@
     </row>
     <row r="143" spans="1:14">
       <c r="A143" s="0">
-        <v>49535653</v>
+        <v>49636184</v>
       </c>
       <c r="B143" s="0" t="inlineStr">
         <is>
-          <t>如意家电13368134456维修</t>
+          <t>古道西风</t>
         </is>
       </c>
       <c r="C143" s="0" t="inlineStr">
@@ -8619,7 +8624,7 @@
       </c>
       <c r="G143" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:28:25</t>
+          <t>2026-08-25 13:18:55</t>
         </is>
       </c>
       <c r="H143" s="0" t="inlineStr">
@@ -8629,7 +8634,7 @@
       </c>
       <c r="I143" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J143" s="0" t="inlineStr">
@@ -8650,11 +8655,11 @@
     </row>
     <row r="144" spans="1:14">
       <c r="A144" s="0">
-        <v>49535650</v>
+        <v>49636170</v>
       </c>
       <c r="B144" s="0" t="inlineStr">
         <is>
-          <t>莺莺</t>
+          <t>周海龙</t>
         </is>
       </c>
       <c r="C144" s="0" t="inlineStr">
@@ -8679,7 +8684,7 @@
       </c>
       <c r="G144" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:27:55</t>
+          <t>2026-08-25 13:18:33</t>
         </is>
       </c>
       <c r="H144" s="0" t="inlineStr">
@@ -8689,7 +8694,7 @@
       </c>
       <c r="I144" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J144" s="0" t="inlineStr">
@@ -8705,21 +8710,16 @@
       <c r="L144" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N144" s="0" t="inlineStr">
-        <is>
-          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="145" spans="1:14">
       <c r="A145" s="0">
-        <v>49508265</v>
+        <v>49636157</v>
       </c>
       <c r="B145" s="0" t="inlineStr">
         <is>
-          <t>爱猫🐱 咪</t>
+          <t>锦妍</t>
         </is>
       </c>
       <c r="C145" s="0" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="G145" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 09:53:41</t>
+          <t>2026-08-25 13:18:07</t>
         </is>
       </c>
       <c r="H145" s="0" t="inlineStr">
@@ -8754,7 +8754,7 @@
       </c>
       <c r="I145" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J145" s="0" t="inlineStr">
@@ -8775,11 +8775,11 @@
     </row>
     <row r="146" spans="1:14">
       <c r="A146" s="0">
-        <v>49493414</v>
+        <v>49593974</v>
       </c>
       <c r="B146" s="0" t="inlineStr">
         <is>
-          <t>惠平</t>
+          <t>兰兰</t>
         </is>
       </c>
       <c r="C146" s="0" t="inlineStr">
@@ -8804,7 +8804,7 @@
       </c>
       <c r="G146" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:53:02</t>
+          <t>2026-08-24 12:59:53</t>
         </is>
       </c>
       <c r="H146" s="0" t="inlineStr">
@@ -8835,11 +8835,11 @@
     </row>
     <row r="147" spans="1:14">
       <c r="A147" s="0">
-        <v>49493126</v>
+        <v>49593671</v>
       </c>
       <c r="B147" s="0" t="inlineStr">
         <is>
-          <t>刘盼昭</t>
+          <t>准备1号</t>
         </is>
       </c>
       <c r="C147" s="0" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="G147" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:44:53</t>
+          <t>2026-08-24 12:49:27</t>
         </is>
       </c>
       <c r="H147" s="0" t="inlineStr">
@@ -8895,11 +8895,11 @@
     </row>
     <row r="148" spans="1:14">
       <c r="A148" s="0">
-        <v>49492499</v>
+        <v>49535916</v>
       </c>
       <c r="B148" s="0" t="inlineStr">
         <is>
-          <t>红霞</t>
+          <t>真诚</t>
         </is>
       </c>
       <c r="C148" s="0" t="inlineStr">
@@ -8924,7 +8924,7 @@
       </c>
       <c r="G148" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:29:43</t>
+          <t>2026-08-22 23:46:23</t>
         </is>
       </c>
       <c r="H148" s="0" t="inlineStr">
@@ -8955,11 +8955,11 @@
     </row>
     <row r="149" spans="1:14">
       <c r="A149" s="0">
-        <v>49455301</v>
+        <v>49535653</v>
       </c>
       <c r="B149" s="0" t="inlineStr">
         <is>
-          <t>周开平</t>
+          <t>如意家电13368134456维修</t>
         </is>
       </c>
       <c r="C149" s="0" t="inlineStr">
@@ -8984,7 +8984,7 @@
       </c>
       <c r="G149" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 22:46:59</t>
+          <t>2026-08-22 23:28:25</t>
         </is>
       </c>
       <c r="H149" s="0" t="inlineStr">
@@ -9015,11 +9015,11 @@
     </row>
     <row r="150" spans="1:14">
       <c r="A150" s="0">
-        <v>49432023</v>
+        <v>49535650</v>
       </c>
       <c r="B150" s="0" t="inlineStr">
         <is>
-          <t>花生米</t>
+          <t>莺莺</t>
         </is>
       </c>
       <c r="C150" s="0" t="inlineStr">
@@ -9044,7 +9044,7 @@
       </c>
       <c r="G150" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 11:55:45</t>
+          <t>2026-08-22 23:27:55</t>
         </is>
       </c>
       <c r="H150" s="0" t="inlineStr">
@@ -9070,16 +9070,21 @@
       <c r="L150" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N150" s="0" t="inlineStr">
+        <is>
+          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="151" spans="1:14">
       <c r="A151" s="0">
-        <v>49415939</v>
+        <v>49508265</v>
       </c>
       <c r="B151" s="0" t="inlineStr">
         <is>
-          <t>杨梅芳</t>
+          <t>爱猫🐱 咪</t>
         </is>
       </c>
       <c r="C151" s="0" t="inlineStr">
@@ -9104,7 +9109,7 @@
       </c>
       <c r="G151" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:58</t>
+          <t>2026-08-22 09:53:41</t>
         </is>
       </c>
       <c r="H151" s="0" t="inlineStr">
@@ -9114,17 +9119,17 @@
       </c>
       <c r="I151" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J151" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K151" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L151" s="0" t="inlineStr">
@@ -9135,11 +9140,11 @@
     </row>
     <row r="152" spans="1:14">
       <c r="A152" s="0">
-        <v>49415918</v>
+        <v>49493414</v>
       </c>
       <c r="B152" s="0" t="inlineStr">
         <is>
-          <t>心语无言</t>
+          <t>惠平</t>
         </is>
       </c>
       <c r="C152" s="0" t="inlineStr">
@@ -9164,7 +9169,7 @@
       </c>
       <c r="G152" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:24</t>
+          <t>2026-08-21 22:53:02</t>
         </is>
       </c>
       <c r="H152" s="0" t="inlineStr">
@@ -9174,17 +9179,17 @@
       </c>
       <c r="I152" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J152" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K152" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L152" s="0" t="inlineStr">
@@ -9195,11 +9200,11 @@
     </row>
     <row r="153" spans="1:14">
       <c r="A153" s="0">
-        <v>49415913</v>
+        <v>49493126</v>
       </c>
       <c r="B153" s="0" t="inlineStr">
         <is>
-          <t>安好</t>
+          <t>刘盼昭</t>
         </is>
       </c>
       <c r="C153" s="0" t="inlineStr">
@@ -9224,7 +9229,7 @@
       </c>
       <c r="G153" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:18</t>
+          <t>2026-08-21 22:44:53</t>
         </is>
       </c>
       <c r="H153" s="0" t="inlineStr">
@@ -9234,17 +9239,17 @@
       </c>
       <c r="I153" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J153" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K153" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L153" s="0" t="inlineStr">
@@ -9255,11 +9260,11 @@
     </row>
     <row r="154" spans="1:14">
       <c r="A154" s="0">
-        <v>49415890</v>
+        <v>49492499</v>
       </c>
       <c r="B154" s="0" t="inlineStr">
         <is>
-          <t>雨夜聆风</t>
+          <t>红霞</t>
         </is>
       </c>
       <c r="C154" s="0" t="inlineStr">
@@ -9284,7 +9289,7 @@
       </c>
       <c r="G154" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:56</t>
+          <t>2026-08-21 22:29:43</t>
         </is>
       </c>
       <c r="H154" s="0" t="inlineStr">
@@ -9294,37 +9299,32 @@
       </c>
       <c r="I154" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J154" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K154" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L154" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N154" s="0" t="inlineStr">
-        <is>
-          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="155" spans="1:14">
       <c r="A155" s="0">
-        <v>49415874</v>
+        <v>49455301</v>
       </c>
       <c r="B155" s="0" t="inlineStr">
         <is>
-          <t>飘</t>
+          <t>周开平</t>
         </is>
       </c>
       <c r="C155" s="0" t="inlineStr">
@@ -9349,7 +9349,7 @@
       </c>
       <c r="G155" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:40</t>
+          <t>2026-08-20 22:46:59</t>
         </is>
       </c>
       <c r="H155" s="0" t="inlineStr">
@@ -9359,17 +9359,17 @@
       </c>
       <c r="I155" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J155" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K155" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L155" s="0" t="inlineStr">
@@ -9380,11 +9380,11 @@
     </row>
     <row r="156" spans="1:14">
       <c r="A156" s="0">
-        <v>49415871</v>
+        <v>49432023</v>
       </c>
       <c r="B156" s="0" t="inlineStr">
         <is>
-          <t>庆</t>
+          <t>花生米</t>
         </is>
       </c>
       <c r="C156" s="0" t="inlineStr">
@@ -9409,7 +9409,7 @@
       </c>
       <c r="G156" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:36</t>
+          <t>2026-08-20 11:55:45</t>
         </is>
       </c>
       <c r="H156" s="0" t="inlineStr">
@@ -9419,17 +9419,17 @@
       </c>
       <c r="I156" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J156" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K156" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L156" s="0" t="inlineStr">
@@ -9440,59 +9440,424 @@
     </row>
     <row r="157" spans="1:14">
       <c r="A157" s="0">
+        <v>49415939</v>
+      </c>
+      <c r="B157" s="0" t="inlineStr">
+        <is>
+          <t>杨梅芳</t>
+        </is>
+      </c>
+      <c r="C157" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D157" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E157" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F157" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G157" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:58</t>
+        </is>
+      </c>
+      <c r="H157" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I157" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J157" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K157" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L157" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" spans="1:14">
+      <c r="A158" s="0">
+        <v>49415918</v>
+      </c>
+      <c r="B158" s="0" t="inlineStr">
+        <is>
+          <t>心语无言</t>
+        </is>
+      </c>
+      <c r="C158" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D158" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E158" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F158" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G158" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:24</t>
+        </is>
+      </c>
+      <c r="H158" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I158" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J158" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K158" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L158" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" spans="1:14">
+      <c r="A159" s="0">
+        <v>49415913</v>
+      </c>
+      <c r="B159" s="0" t="inlineStr">
+        <is>
+          <t>安好</t>
+        </is>
+      </c>
+      <c r="C159" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D159" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E159" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F159" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G159" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:48:18</t>
+        </is>
+      </c>
+      <c r="H159" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I159" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J159" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K159" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L159" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" spans="1:14">
+      <c r="A160" s="0">
+        <v>49415890</v>
+      </c>
+      <c r="B160" s="0" t="inlineStr">
+        <is>
+          <t>雨夜聆风</t>
+        </is>
+      </c>
+      <c r="C160" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D160" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E160" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F160" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G160" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:56</t>
+        </is>
+      </c>
+      <c r="H160" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I160" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J160" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K160" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L160" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+      <c r="N160" s="0" t="inlineStr">
+        <is>
+          <t>宜春</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" spans="1:14">
+      <c r="A161" s="0">
+        <v>49415874</v>
+      </c>
+      <c r="B161" s="0" t="inlineStr">
+        <is>
+          <t>飘</t>
+        </is>
+      </c>
+      <c r="C161" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D161" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E161" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F161" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G161" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:40</t>
+        </is>
+      </c>
+      <c r="H161" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I161" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J161" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K161" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L161" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" spans="1:14">
+      <c r="A162" s="0">
+        <v>49415871</v>
+      </c>
+      <c r="B162" s="0" t="inlineStr">
+        <is>
+          <t>庆</t>
+        </is>
+      </c>
+      <c r="C162" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D162" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E162" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F162" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G162" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:36</t>
+        </is>
+      </c>
+      <c r="H162" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I162" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J162" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K162" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L162" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" spans="1:14">
+      <c r="A163" s="0">
         <v>49415867</v>
       </c>
-      <c r="B157" s="0" t="inlineStr">
+      <c r="B163" s="0" t="inlineStr">
         <is>
           <t>HYQ</t>
         </is>
       </c>
-      <c r="C157" s="0" t="inlineStr">
-        <is>
-          <t>6天0基础钢琴入门课</t>
-        </is>
-      </c>
-      <c r="D157" s="0" t="inlineStr">
-        <is>
-          <t>训练营</t>
-        </is>
-      </c>
-      <c r="E157" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="F157" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="G157" s="0" t="inlineStr">
+      <c r="C163" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D163" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E163" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F163" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G163" s="0" t="inlineStr">
         <is>
           <t>2026-08-19 22:47:33</t>
         </is>
       </c>
-      <c r="H157" s="0" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I157" s="0" t="inlineStr">
-        <is>
-          <t>黄老师-抖音01</t>
-        </is>
-      </c>
-      <c r="J157" s="0" t="inlineStr">
+      <c r="H163" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I163" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J163" s="0" t="inlineStr">
         <is>
           <t>安迪钢琴-多个点击报名-0元</t>
         </is>
       </c>
-      <c r="K157" s="0" t="inlineStr">
+      <c r="K163" s="0" t="inlineStr">
         <is>
           <t>微信支付</t>
         </is>
       </c>
-      <c r="L157" s="0" t="inlineStr">
+      <c r="L163" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>

</xml_diff>

<commit_message>
📅 日报更新 2026-09-06 11:06
</commit_message>
<xml_diff>
--- a/data/exports/黄老师/dist_order_2026-09-06.xlsx
+++ b/data/exports/黄老师/dist_order_2026-09-06.xlsx
@@ -125,11 +125,11 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="0">
-        <v>50121359</v>
+        <v>50129606</v>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>amy</t>
+          <t>A1风轻云淡</t>
         </is>
       </c>
       <c r="C2" s="0" t="inlineStr">
@@ -154,7 +154,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 12:58:35</t>
+          <t>2026-09-06 17:53:57</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -164,7 +164,7 @@
       </c>
       <c r="I2" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J2" s="0" t="inlineStr">
@@ -185,11 +185,11 @@
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="0">
-        <v>50121001</v>
+        <v>50129482</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>莲花李秀清</t>
+          <t>一心有你电话号码，</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
@@ -214,7 +214,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 12:47:43</t>
+          <t>2026-09-06 17:49:45</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -224,7 +224,7 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J3" s="0" t="inlineStr">
@@ -245,11 +245,11 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="0">
-        <v>50120862</v>
+        <v>50121359</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>cobra</t>
+          <t>amy</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
@@ -274,7 +274,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 12:44:33</t>
+          <t>2026-09-06 12:58:35</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -284,7 +284,7 @@
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J4" s="0" t="inlineStr">
@@ -305,11 +305,11 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="0">
-        <v>50120856</v>
+        <v>50121001</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>海边的星空</t>
+          <t>莲花李秀清</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
@@ -334,7 +334,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 12:44:17</t>
+          <t>2026-09-06 12:47:43</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -344,7 +344,7 @@
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J5" s="0" t="inlineStr">
@@ -365,11 +365,11 @@
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="0">
-        <v>50120852</v>
+        <v>50120862</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>柠檬黄🍋陈</t>
+          <t>cobra</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -394,7 +394,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 12:44:09</t>
+          <t>2026-09-06 12:44:33</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -425,11 +425,11 @@
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="0">
-        <v>50120848</v>
+        <v>50120856</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>英子</t>
+          <t>海边的星空</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 12:44:01</t>
+          <t>2026-09-06 12:44:17</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -485,11 +485,11 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="0">
-        <v>50120818</v>
+        <v>50120852</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>peaceful</t>
+          <t>柠檬黄🍋陈</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 12:42:49</t>
+          <t>2026-09-06 12:44:09</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -545,11 +545,11 @@
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="0">
-        <v>50120817</v>
+        <v>50120848</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>fj</t>
+          <t>英子</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 12:42:49</t>
+          <t>2026-09-06 12:44:01</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -605,11 +605,11 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="0">
-        <v>50120806</v>
+        <v>50120818</v>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>💍小薇🎀💎🌷</t>
+          <t>peaceful</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 12:42:27</t>
+          <t>2026-09-06 12:42:49</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
@@ -665,11 +665,11 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="0">
-        <v>50120803</v>
+        <v>50120817</v>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>于小毛</t>
+          <t>fj</t>
         </is>
       </c>
       <c r="C11" s="0" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 12:42:25</t>
+          <t>2026-09-06 12:42:49</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -725,11 +725,11 @@
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="0">
-        <v>50116869</v>
+        <v>50120806</v>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>美义</t>
+          <t>💍小薇🎀💎🌷</t>
         </is>
       </c>
       <c r="C12" s="0" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="G12" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 10:56:33</t>
+          <t>2026-09-06 12:42:27</t>
         </is>
       </c>
       <c r="H12" s="0" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="I12" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J12" s="0" t="inlineStr">
@@ -785,11 +785,11 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="0">
-        <v>50114006</v>
+        <v>50120803</v>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>幸运草</t>
+          <t>于小毛</t>
         </is>
       </c>
       <c r="C13" s="0" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 09:45:01</t>
+          <t>2026-09-06 12:42:25</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
@@ -845,11 +845,11 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="0">
-        <v>50113664</v>
+        <v>50116869</v>
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>执子之手</t>
+          <t>美义</t>
         </is>
       </c>
       <c r="C14" s="0" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 09:37:35</t>
+          <t>2026-09-06 10:56:33</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="I14" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J14" s="0" t="inlineStr">
@@ -905,11 +905,11 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="0">
-        <v>50113641</v>
+        <v>50114006</v>
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>新视野</t>
+          <t>幸运草</t>
         </is>
       </c>
       <c r="C15" s="0" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 09:36:52</t>
+          <t>2026-09-06 09:45:01</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -965,11 +965,11 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="0">
-        <v>50113640</v>
+        <v>50113664</v>
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>安静且聆听</t>
+          <t>执子之手</t>
         </is>
       </c>
       <c r="C16" s="0" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 09:36:49</t>
+          <t>2026-09-06 09:37:35</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
@@ -1020,21 +1020,16 @@
       <c r="L16" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N16" s="0" t="inlineStr">
-        <is>
-          <t>保山</t>
         </is>
       </c>
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="0">
-        <v>50113638</v>
+        <v>50113641</v>
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>十月</t>
+          <t>新视野</t>
         </is>
       </c>
       <c r="C17" s="0" t="inlineStr">
@@ -1059,7 +1054,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>2026-09-06 09:36:45</t>
+          <t>2026-09-06 09:36:52</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
@@ -1090,11 +1085,11 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="0">
-        <v>50100338</v>
+        <v>50113640</v>
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>青山绿水</t>
+          <t>安静且聆听</t>
         </is>
       </c>
       <c r="C18" s="0" t="inlineStr">
@@ -1119,7 +1114,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 23:10:04</t>
+          <t>2026-09-06 09:36:49</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
@@ -1145,16 +1140,21 @@
       <c r="L18" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N18" s="0" t="inlineStr">
+        <is>
+          <t>保山</t>
         </is>
       </c>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="0">
-        <v>50100035</v>
+        <v>50113638</v>
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>杨</t>
+          <t>十月</t>
         </is>
       </c>
       <c r="C19" s="0" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:57:53</t>
+          <t>2026-09-06 09:36:45</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="I19" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J19" s="0" t="inlineStr">
@@ -1210,11 +1210,11 @@
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="0">
-        <v>50100033</v>
+        <v>50100338</v>
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>雨后彩虹</t>
+          <t>青山绿水</t>
         </is>
       </c>
       <c r="C20" s="0" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:57:47</t>
+          <t>2026-09-05 23:10:04</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="I20" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J20" s="0" t="inlineStr">
@@ -1270,11 +1270,11 @@
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="0">
-        <v>50100028</v>
+        <v>50100035</v>
       </c>
       <c r="B21" s="0" t="inlineStr">
         <is>
-          <t>首信海报</t>
+          <t>杨</t>
         </is>
       </c>
       <c r="C21" s="0" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:57:32</t>
+          <t>2026-09-05 22:57:53</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
@@ -1330,11 +1330,11 @@
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="0">
-        <v>50099958</v>
+        <v>50100033</v>
       </c>
       <c r="B22" s="0" t="inlineStr">
         <is>
-          <t>张君</t>
+          <t>雨后彩虹</t>
         </is>
       </c>
       <c r="C22" s="0" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:55:57</t>
+          <t>2026-09-05 22:57:47</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
@@ -1390,11 +1390,11 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="0">
-        <v>50099933</v>
+        <v>50100028</v>
       </c>
       <c r="B23" s="0" t="inlineStr">
         <is>
-          <t>耶和华以勒</t>
+          <t>首信海报</t>
         </is>
       </c>
       <c r="C23" s="0" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:55:31</t>
+          <t>2026-09-05 22:57:32</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
@@ -1450,11 +1450,11 @@
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="0">
-        <v>50099844</v>
+        <v>50099958</v>
       </c>
       <c r="B24" s="0" t="inlineStr">
         <is>
-          <t>平安</t>
+          <t>张君</t>
         </is>
       </c>
       <c r="C24" s="0" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="G24" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:51:49</t>
+          <t>2026-09-05 22:55:57</t>
         </is>
       </c>
       <c r="H24" s="0" t="inlineStr">
@@ -1510,11 +1510,11 @@
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="0">
-        <v>50099768</v>
+        <v>50099933</v>
       </c>
       <c r="B25" s="0" t="inlineStr">
         <is>
-          <t>阳</t>
+          <t>耶和华以勒</t>
         </is>
       </c>
       <c r="C25" s="0" t="inlineStr">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:49:01</t>
+          <t>2026-09-05 22:55:31</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="I25" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J25" s="0" t="inlineStr">
@@ -1570,11 +1570,11 @@
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="0">
-        <v>50099767</v>
+        <v>50099844</v>
       </c>
       <c r="B26" s="0" t="inlineStr">
         <is>
-          <t>梦&amp;爷💫</t>
+          <t>平安</t>
         </is>
       </c>
       <c r="C26" s="0" t="inlineStr">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:57</t>
+          <t>2026-09-05 22:51:49</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="I26" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J26" s="0" t="inlineStr">
@@ -1630,11 +1630,11 @@
     </row>
     <row r="27" spans="1:14">
       <c r="A27" s="0">
-        <v>50099763</v>
+        <v>50099768</v>
       </c>
       <c r="B27" s="0" t="inlineStr">
         <is>
-          <t>李丽</t>
+          <t>阳</t>
         </is>
       </c>
       <c r="C27" s="0" t="inlineStr">
@@ -1659,7 +1659,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:53</t>
+          <t>2026-09-05 22:49:01</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
@@ -1690,11 +1690,11 @@
     </row>
     <row r="28" spans="1:14">
       <c r="A28" s="0">
-        <v>50099760</v>
+        <v>50099767</v>
       </c>
       <c r="B28" s="0" t="inlineStr">
         <is>
-          <t>A选择无悔</t>
+          <t>梦&amp;爷💫</t>
         </is>
       </c>
       <c r="C28" s="0" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:46</t>
+          <t>2026-09-05 22:48:57</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
@@ -1750,11 +1750,11 @@
     </row>
     <row r="29" spans="1:14">
       <c r="A29" s="0">
-        <v>50099759</v>
+        <v>50099763</v>
       </c>
       <c r="B29" s="0" t="inlineStr">
         <is>
-          <t>信念</t>
+          <t>李丽</t>
         </is>
       </c>
       <c r="C29" s="0" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:44</t>
+          <t>2026-09-05 22:48:53</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
@@ -1810,11 +1810,11 @@
     </row>
     <row r="30" spans="1:14">
       <c r="A30" s="0">
-        <v>50099757</v>
+        <v>50099760</v>
       </c>
       <c r="B30" s="0" t="inlineStr">
         <is>
-          <t>李lee</t>
+          <t>A选择无悔</t>
         </is>
       </c>
       <c r="C30" s="0" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:41</t>
+          <t>2026-09-05 22:48:46</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
@@ -1870,11 +1870,11 @@
     </row>
     <row r="31" spans="1:14">
       <c r="A31" s="0">
-        <v>50099755</v>
+        <v>50099759</v>
       </c>
       <c r="B31" s="0" t="inlineStr">
         <is>
-          <t>徐飛燕*^O^*</t>
+          <t>信念</t>
         </is>
       </c>
       <c r="C31" s="0" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="G31" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:39</t>
+          <t>2026-09-05 22:48:44</t>
         </is>
       </c>
       <c r="H31" s="0" t="inlineStr">
@@ -1930,11 +1930,11 @@
     </row>
     <row r="32" spans="1:14">
       <c r="A32" s="0">
-        <v>50099752</v>
+        <v>50099757</v>
       </c>
       <c r="B32" s="0" t="inlineStr">
         <is>
-          <t>星移*</t>
+          <t>李lee</t>
         </is>
       </c>
       <c r="C32" s="0" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="G32" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:35</t>
+          <t>2026-09-05 22:48:41</t>
         </is>
       </c>
       <c r="H32" s="0" t="inlineStr">
@@ -1990,11 +1990,11 @@
     </row>
     <row r="33" spans="1:14">
       <c r="A33" s="0">
-        <v>50099749</v>
+        <v>50099755</v>
       </c>
       <c r="B33" s="0" t="inlineStr">
         <is>
-          <t>刘勇</t>
+          <t>徐飛燕*^O^*</t>
         </is>
       </c>
       <c r="C33" s="0" t="inlineStr">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:28</t>
+          <t>2026-09-05 22:48:39</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
@@ -2050,11 +2050,11 @@
     </row>
     <row r="34" spans="1:14">
       <c r="A34" s="0">
-        <v>50099741</v>
+        <v>50099752</v>
       </c>
       <c r="B34" s="0" t="inlineStr">
         <is>
-          <t>碧皓之游</t>
+          <t>星移*</t>
         </is>
       </c>
       <c r="C34" s="0" t="inlineStr">
@@ -2079,7 +2079,7 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:15</t>
+          <t>2026-09-05 22:48:35</t>
         </is>
       </c>
       <c r="H34" s="0" t="inlineStr">
@@ -2110,11 +2110,11 @@
     </row>
     <row r="35" spans="1:14">
       <c r="A35" s="0">
-        <v>50099737</v>
+        <v>50099749</v>
       </c>
       <c r="B35" s="0" t="inlineStr">
         <is>
-          <t>书心燕语</t>
+          <t>刘勇</t>
         </is>
       </c>
       <c r="C35" s="0" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:48:03</t>
+          <t>2026-09-05 22:48:28</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
@@ -2170,11 +2170,11 @@
     </row>
     <row r="36" spans="1:14">
       <c r="A36" s="0">
-        <v>50099733</v>
+        <v>50099741</v>
       </c>
       <c r="B36" s="0" t="inlineStr">
         <is>
-          <t>ღ᭄ꦿ微微一笑ღ᭄ꦿ</t>
+          <t>碧皓之游</t>
         </is>
       </c>
       <c r="C36" s="0" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 22:47:47</t>
+          <t>2026-09-05 22:48:15</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
@@ -2230,11 +2230,11 @@
     </row>
     <row r="37" spans="1:14">
       <c r="A37" s="0">
-        <v>50080657</v>
+        <v>50099737</v>
       </c>
       <c r="B37" s="0" t="inlineStr">
         <is>
-          <t>平红</t>
+          <t>书心燕语</t>
         </is>
       </c>
       <c r="C37" s="0" t="inlineStr">
@@ -2259,7 +2259,7 @@
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:07:13</t>
+          <t>2026-09-05 22:48:03</t>
         </is>
       </c>
       <c r="H37" s="0" t="inlineStr">
@@ -2290,11 +2290,11 @@
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="0">
-        <v>50080582</v>
+        <v>50099733</v>
       </c>
       <c r="B38" s="0" t="inlineStr">
         <is>
-          <t>aabb</t>
+          <t>ღ᭄ꦿ微微一笑ღ᭄ꦿ</t>
         </is>
       </c>
       <c r="C38" s="0" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:05:19</t>
+          <t>2026-09-05 22:47:47</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
@@ -2350,11 +2350,11 @@
     </row>
     <row r="39" spans="1:14">
       <c r="A39" s="0">
-        <v>50080559</v>
+        <v>50080657</v>
       </c>
       <c r="B39" s="0" t="inlineStr">
         <is>
-          <t>自由人</t>
+          <t>平红</t>
         </is>
       </c>
       <c r="C39" s="0" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:04:28</t>
+          <t>2026-09-05 13:07:13</t>
         </is>
       </c>
       <c r="H39" s="0" t="inlineStr">
@@ -2410,11 +2410,11 @@
     </row>
     <row r="40" spans="1:14">
       <c r="A40" s="0">
-        <v>50080553</v>
+        <v>50080582</v>
       </c>
       <c r="B40" s="0" t="inlineStr">
         <is>
-          <t>晶晶</t>
+          <t>aabb</t>
         </is>
       </c>
       <c r="C40" s="0" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="G40" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:04:15</t>
+          <t>2026-09-05 13:05:19</t>
         </is>
       </c>
       <c r="H40" s="0" t="inlineStr">
@@ -2470,11 +2470,11 @@
     </row>
     <row r="41" spans="1:14">
       <c r="A41" s="0">
-        <v>50080549</v>
+        <v>50080559</v>
       </c>
       <c r="B41" s="0" t="inlineStr">
         <is>
-          <t>abc</t>
+          <t>自由人</t>
         </is>
       </c>
       <c r="C41" s="0" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:04:09</t>
+          <t>2026-09-05 13:04:28</t>
         </is>
       </c>
       <c r="H41" s="0" t="inlineStr">
@@ -2530,11 +2530,11 @@
     </row>
     <row r="42" spans="1:14">
       <c r="A42" s="0">
-        <v>50080548</v>
+        <v>50080553</v>
       </c>
       <c r="B42" s="0" t="inlineStr">
         <is>
-          <t>盘子</t>
+          <t>晶晶</t>
         </is>
       </c>
       <c r="C42" s="0" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:04:08</t>
+          <t>2026-09-05 13:04:15</t>
         </is>
       </c>
       <c r="H42" s="0" t="inlineStr">
@@ -2590,11 +2590,11 @@
     </row>
     <row r="43" spans="1:14">
       <c r="A43" s="0">
-        <v>50080547</v>
+        <v>50080549</v>
       </c>
       <c r="B43" s="0" t="inlineStr">
         <is>
-          <t>赵满珍C5</t>
+          <t>abc</t>
         </is>
       </c>
       <c r="C43" s="0" t="inlineStr">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:04:05</t>
+          <t>2026-09-05 13:04:09</t>
         </is>
       </c>
       <c r="H43" s="0" t="inlineStr">
@@ -2650,11 +2650,11 @@
     </row>
     <row r="44" spans="1:14">
       <c r="A44" s="0">
-        <v>50080539</v>
+        <v>50080548</v>
       </c>
       <c r="B44" s="0" t="inlineStr">
         <is>
-          <t>平平安安</t>
+          <t>盘子</t>
         </is>
       </c>
       <c r="C44" s="0" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:51</t>
+          <t>2026-09-05 13:04:08</t>
         </is>
       </c>
       <c r="H44" s="0" t="inlineStr">
@@ -2710,11 +2710,11 @@
     </row>
     <row r="45" spans="1:14">
       <c r="A45" s="0">
-        <v>50080538</v>
+        <v>50080547</v>
       </c>
       <c r="B45" s="0" t="inlineStr">
         <is>
-          <t>凡事包容</t>
+          <t>赵满珍C5</t>
         </is>
       </c>
       <c r="C45" s="0" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="G45" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:51</t>
+          <t>2026-09-05 13:04:05</t>
         </is>
       </c>
       <c r="H45" s="0" t="inlineStr">
@@ -2770,11 +2770,11 @@
     </row>
     <row r="46" spans="1:14">
       <c r="A46" s="0">
-        <v>50080536</v>
+        <v>50080539</v>
       </c>
       <c r="B46" s="0" t="inlineStr">
         <is>
-          <t>吴忧无忧</t>
+          <t>平平安安</t>
         </is>
       </c>
       <c r="C46" s="0" t="inlineStr">
@@ -2799,7 +2799,7 @@
       </c>
       <c r="G46" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:47</t>
+          <t>2026-09-05 13:03:51</t>
         </is>
       </c>
       <c r="H46" s="0" t="inlineStr">
@@ -2830,11 +2830,11 @@
     </row>
     <row r="47" spans="1:14">
       <c r="A47" s="0">
-        <v>50080535</v>
+        <v>50080538</v>
       </c>
       <c r="B47" s="0" t="inlineStr">
         <is>
-          <t>小鱼儿</t>
+          <t>凡事包容</t>
         </is>
       </c>
       <c r="C47" s="0" t="inlineStr">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="G47" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:43</t>
+          <t>2026-09-05 13:03:51</t>
         </is>
       </c>
       <c r="H47" s="0" t="inlineStr">
@@ -2890,11 +2890,11 @@
     </row>
     <row r="48" spans="1:14">
       <c r="A48" s="0">
-        <v>50080525</v>
+        <v>50080536</v>
       </c>
       <c r="B48" s="0" t="inlineStr">
         <is>
-          <t>辞芝锦😎</t>
+          <t>吴忧无忧</t>
         </is>
       </c>
       <c r="C48" s="0" t="inlineStr">
@@ -2919,7 +2919,7 @@
       </c>
       <c r="G48" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:29</t>
+          <t>2026-09-05 13:03:47</t>
         </is>
       </c>
       <c r="H48" s="0" t="inlineStr">
@@ -2950,11 +2950,11 @@
     </row>
     <row r="49" spans="1:14">
       <c r="A49" s="0">
-        <v>50080523</v>
+        <v>50080535</v>
       </c>
       <c r="B49" s="0" t="inlineStr">
         <is>
-          <t>早陈</t>
+          <t>小鱼儿</t>
         </is>
       </c>
       <c r="C49" s="0" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="G49" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:21</t>
+          <t>2026-09-05 13:03:43</t>
         </is>
       </c>
       <c r="H49" s="0" t="inlineStr">
@@ -3010,11 +3010,11 @@
     </row>
     <row r="50" spans="1:14">
       <c r="A50" s="0">
-        <v>50080516</v>
+        <v>50080525</v>
       </c>
       <c r="B50" s="0" t="inlineStr">
         <is>
-          <t>星星の恋人</t>
+          <t>辞芝锦😎</t>
         </is>
       </c>
       <c r="C50" s="0" t="inlineStr">
@@ -3039,7 +3039,7 @@
       </c>
       <c r="G50" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:13</t>
+          <t>2026-09-05 13:03:29</t>
         </is>
       </c>
       <c r="H50" s="0" t="inlineStr">
@@ -3070,11 +3070,11 @@
     </row>
     <row r="51" spans="1:14">
       <c r="A51" s="0">
-        <v>50080511</v>
+        <v>50080523</v>
       </c>
       <c r="B51" s="0" t="inlineStr">
         <is>
-          <t>无咎</t>
+          <t>早陈</t>
         </is>
       </c>
       <c r="C51" s="0" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="G51" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:03:09</t>
+          <t>2026-09-05 13:03:21</t>
         </is>
       </c>
       <c r="H51" s="0" t="inlineStr">
@@ -3130,11 +3130,11 @@
     </row>
     <row r="52" spans="1:14">
       <c r="A52" s="0">
-        <v>50080477</v>
+        <v>50080516</v>
       </c>
       <c r="B52" s="0" t="inlineStr">
         <is>
-          <t>刘小虎</t>
+          <t>星星の恋人</t>
         </is>
       </c>
       <c r="C52" s="0" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="G52" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 13:02:37</t>
+          <t>2026-09-05 13:03:13</t>
         </is>
       </c>
       <c r="H52" s="0" t="inlineStr">
@@ -3190,11 +3190,11 @@
     </row>
     <row r="53" spans="1:14">
       <c r="A53" s="0">
-        <v>50074867</v>
+        <v>50080511</v>
       </c>
       <c r="B53" s="0" t="inlineStr">
         <is>
-          <t>美好人生</t>
+          <t>无咎</t>
         </is>
       </c>
       <c r="C53" s="0" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="G53" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 10:19:59</t>
+          <t>2026-09-05 13:03:09</t>
         </is>
       </c>
       <c r="H53" s="0" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="I53" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J53" s="0" t="inlineStr">
@@ -3250,11 +3250,11 @@
     </row>
     <row r="54" spans="1:14">
       <c r="A54" s="0">
-        <v>50074273</v>
+        <v>50080477</v>
       </c>
       <c r="B54" s="0" t="inlineStr">
         <is>
-          <t>周利平</t>
+          <t>刘小虎</t>
         </is>
       </c>
       <c r="C54" s="0" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="G54" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 10:02:26</t>
+          <t>2026-09-05 13:02:37</t>
         </is>
       </c>
       <c r="H54" s="0" t="inlineStr">
@@ -3310,11 +3310,11 @@
     </row>
     <row r="55" spans="1:14">
       <c r="A55" s="0">
-        <v>50074103</v>
+        <v>50074867</v>
       </c>
       <c r="B55" s="0" t="inlineStr">
         <is>
-          <t>赵香荣</t>
+          <t>美好人生</t>
         </is>
       </c>
       <c r="C55" s="0" t="inlineStr">
@@ -3339,7 +3339,7 @@
       </c>
       <c r="G55" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:58:29</t>
+          <t>2026-09-05 10:19:59</t>
         </is>
       </c>
       <c r="H55" s="0" t="inlineStr">
@@ -3349,7 +3349,7 @@
       </c>
       <c r="I55" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J55" s="0" t="inlineStr">
@@ -3370,11 +3370,11 @@
     </row>
     <row r="56" spans="1:14">
       <c r="A56" s="0">
-        <v>50074078</v>
+        <v>50074273</v>
       </c>
       <c r="B56" s="0" t="inlineStr">
         <is>
-          <t>长风渡℡明</t>
+          <t>周利平</t>
         </is>
       </c>
       <c r="C56" s="0" t="inlineStr">
@@ -3399,7 +3399,7 @@
       </c>
       <c r="G56" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:49</t>
+          <t>2026-09-05 10:02:26</t>
         </is>
       </c>
       <c r="H56" s="0" t="inlineStr">
@@ -3430,11 +3430,11 @@
     </row>
     <row r="57" spans="1:14">
       <c r="A57" s="0">
-        <v>50074077</v>
+        <v>50074103</v>
       </c>
       <c r="B57" s="0" t="inlineStr">
         <is>
-          <t>海阔天空bi</t>
+          <t>赵香荣</t>
         </is>
       </c>
       <c r="C57" s="0" t="inlineStr">
@@ -3459,7 +3459,7 @@
       </c>
       <c r="G57" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:47</t>
+          <t>2026-09-05 09:58:29</t>
         </is>
       </c>
       <c r="H57" s="0" t="inlineStr">
@@ -3490,11 +3490,11 @@
     </row>
     <row r="58" spans="1:14">
       <c r="A58" s="0">
-        <v>50074076</v>
+        <v>50074078</v>
       </c>
       <c r="B58" s="0" t="inlineStr">
         <is>
-          <t>枫叶红</t>
+          <t>长风渡℡明</t>
         </is>
       </c>
       <c r="C58" s="0" t="inlineStr">
@@ -3519,7 +3519,7 @@
       </c>
       <c r="G58" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:47</t>
+          <t>2026-09-05 09:57:49</t>
         </is>
       </c>
       <c r="H58" s="0" t="inlineStr">
@@ -3550,11 +3550,11 @@
     </row>
     <row r="59" spans="1:14">
       <c r="A59" s="0">
-        <v>50074071</v>
+        <v>50074077</v>
       </c>
       <c r="B59" s="0" t="inlineStr">
         <is>
-          <t>思缘</t>
+          <t>海阔天空bi</t>
         </is>
       </c>
       <c r="C59" s="0" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="G59" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:35</t>
+          <t>2026-09-05 09:57:47</t>
         </is>
       </c>
       <c r="H59" s="0" t="inlineStr">
@@ -3610,11 +3610,11 @@
     </row>
     <row r="60" spans="1:14">
       <c r="A60" s="0">
-        <v>50074067</v>
+        <v>50074076</v>
       </c>
       <c r="B60" s="0" t="inlineStr">
         <is>
-          <t>悠然</t>
+          <t>枫叶红</t>
         </is>
       </c>
       <c r="C60" s="0" t="inlineStr">
@@ -3639,7 +3639,7 @@
       </c>
       <c r="G60" s="0" t="inlineStr">
         <is>
-          <t>2026-09-05 09:57:25</t>
+          <t>2026-09-05 09:57:47</t>
         </is>
       </c>
       <c r="H60" s="0" t="inlineStr">
@@ -3670,11 +3670,11 @@
     </row>
     <row r="61" spans="1:14">
       <c r="A61" s="0">
-        <v>50058017</v>
+        <v>50074071</v>
       </c>
       <c r="B61" s="0" t="inlineStr">
         <is>
-          <t>索描贾师＃壹皇贰金山玉旗🇨🇳</t>
+          <t>思缘</t>
         </is>
       </c>
       <c r="C61" s="0" t="inlineStr">
@@ -3699,7 +3699,7 @@
       </c>
       <c r="G61" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:16:49</t>
+          <t>2026-09-05 09:57:35</t>
         </is>
       </c>
       <c r="H61" s="0" t="inlineStr">
@@ -3730,11 +3730,11 @@
     </row>
     <row r="62" spans="1:14">
       <c r="A62" s="0">
-        <v>50057895</v>
+        <v>50074067</v>
       </c>
       <c r="B62" s="0" t="inlineStr">
         <is>
-          <t>南雪</t>
+          <t>悠然</t>
         </is>
       </c>
       <c r="C62" s="0" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="G62" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:12:32</t>
+          <t>2026-09-05 09:57:25</t>
         </is>
       </c>
       <c r="H62" s="0" t="inlineStr">
@@ -3785,21 +3785,16 @@
       <c r="L62" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N62" s="0" t="inlineStr">
-        <is>
-          <t>镇江</t>
         </is>
       </c>
     </row>
     <row r="63" spans="1:14">
       <c r="A63" s="0">
-        <v>50057857</v>
+        <v>50058017</v>
       </c>
       <c r="B63" s="0" t="inlineStr">
         <is>
-          <t>可心</t>
+          <t>索描贾师＃壹皇贰金山玉旗🇨🇳</t>
         </is>
       </c>
       <c r="C63" s="0" t="inlineStr">
@@ -3824,7 +3819,7 @@
       </c>
       <c r="G63" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:55</t>
+          <t>2026-09-04 23:16:49</t>
         </is>
       </c>
       <c r="H63" s="0" t="inlineStr">
@@ -3855,11 +3850,11 @@
     </row>
     <row r="64" spans="1:14">
       <c r="A64" s="0">
-        <v>50057854</v>
+        <v>50057895</v>
       </c>
       <c r="B64" s="0" t="inlineStr">
         <is>
-          <t>张苏龙</t>
+          <t>南雪</t>
         </is>
       </c>
       <c r="C64" s="0" t="inlineStr">
@@ -3884,7 +3879,7 @@
       </c>
       <c r="G64" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:51</t>
+          <t>2026-09-04 23:12:32</t>
         </is>
       </c>
       <c r="H64" s="0" t="inlineStr">
@@ -3910,16 +3905,21 @@
       <c r="L64" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N64" s="0" t="inlineStr">
+        <is>
+          <t>镇江</t>
         </is>
       </c>
     </row>
     <row r="65" spans="1:14">
       <c r="A65" s="0">
-        <v>50057852</v>
+        <v>50057857</v>
       </c>
       <c r="B65" s="0" t="inlineStr">
         <is>
-          <t>？</t>
+          <t>可心</t>
         </is>
       </c>
       <c r="C65" s="0" t="inlineStr">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="G65" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:43</t>
+          <t>2026-09-04 23:10:55</t>
         </is>
       </c>
       <c r="H65" s="0" t="inlineStr">
@@ -3975,11 +3975,11 @@
     </row>
     <row r="66" spans="1:14">
       <c r="A66" s="0">
-        <v>50057841</v>
+        <v>50057854</v>
       </c>
       <c r="B66" s="0" t="inlineStr">
         <is>
-          <t>向往的生活-电信号</t>
+          <t>张苏龙</t>
         </is>
       </c>
       <c r="C66" s="0" t="inlineStr">
@@ -4004,7 +4004,7 @@
       </c>
       <c r="G66" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:09</t>
+          <t>2026-09-04 23:10:51</t>
         </is>
       </c>
       <c r="H66" s="0" t="inlineStr">
@@ -4035,11 +4035,11 @@
     </row>
     <row r="67" spans="1:14">
       <c r="A67" s="0">
-        <v>50057839</v>
+        <v>50057852</v>
       </c>
       <c r="B67" s="0" t="inlineStr">
         <is>
-          <t>金盏花</t>
+          <t>？</t>
         </is>
       </c>
       <c r="C67" s="0" t="inlineStr">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="G67" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 23:10:03</t>
+          <t>2026-09-04 23:10:43</t>
         </is>
       </c>
       <c r="H67" s="0" t="inlineStr">
@@ -4095,11 +4095,11 @@
     </row>
     <row r="68" spans="1:14">
       <c r="A68" s="0">
-        <v>50032697</v>
+        <v>50057841</v>
       </c>
       <c r="B68" s="0" t="inlineStr">
         <is>
-          <t>小米. ᩚ</t>
+          <t>向往的生活-电信号</t>
         </is>
       </c>
       <c r="C68" s="0" t="inlineStr">
@@ -4124,7 +4124,7 @@
       </c>
       <c r="G68" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:24:13</t>
+          <t>2026-09-04 23:10:09</t>
         </is>
       </c>
       <c r="H68" s="0" t="inlineStr">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="I68" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J68" s="0" t="inlineStr">
@@ -4155,11 +4155,11 @@
     </row>
     <row r="69" spans="1:14">
       <c r="A69" s="0">
-        <v>50032693</v>
+        <v>50057839</v>
       </c>
       <c r="B69" s="0" t="inlineStr">
         <is>
-          <t>海岸</t>
+          <t>金盏花</t>
         </is>
       </c>
       <c r="C69" s="0" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="G69" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:24:11</t>
+          <t>2026-09-04 23:10:03</t>
         </is>
       </c>
       <c r="H69" s="0" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="I69" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J69" s="0" t="inlineStr">
@@ -4215,11 +4215,11 @@
     </row>
     <row r="70" spans="1:14">
       <c r="A70" s="0">
-        <v>50032683</v>
+        <v>50032697</v>
       </c>
       <c r="B70" s="0" t="inlineStr">
         <is>
-          <t>陆建军</t>
+          <t>小米. ᩚ</t>
         </is>
       </c>
       <c r="C70" s="0" t="inlineStr">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="G70" s="0" t="inlineStr">
         <is>
-          <t>2026-09-04 12:23:53</t>
+          <t>2026-09-04 12:24:13</t>
         </is>
       </c>
       <c r="H70" s="0" t="inlineStr">
@@ -4275,11 +4275,11 @@
     </row>
     <row r="71" spans="1:14">
       <c r="A71" s="0">
-        <v>50015883</v>
+        <v>50032693</v>
       </c>
       <c r="B71" s="0" t="inlineStr">
         <is>
-          <t>A00金华义乌叉车出租电15268650979</t>
+          <t>海岸</t>
         </is>
       </c>
       <c r="C71" s="0" t="inlineStr">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="G71" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:18:02</t>
+          <t>2026-09-04 12:24:11</t>
         </is>
       </c>
       <c r="H71" s="0" t="inlineStr">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="I71" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J71" s="0" t="inlineStr">
@@ -4335,11 +4335,11 @@
     </row>
     <row r="72" spans="1:14">
       <c r="A72" s="0">
-        <v>50015882</v>
+        <v>50032683</v>
       </c>
       <c r="B72" s="0" t="inlineStr">
         <is>
-          <t>建程仓储中心 张川</t>
+          <t>陆建军</t>
         </is>
       </c>
       <c r="C72" s="0" t="inlineStr">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="G72" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:18:02</t>
+          <t>2026-09-04 12:23:53</t>
         </is>
       </c>
       <c r="H72" s="0" t="inlineStr">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="I72" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J72" s="0" t="inlineStr">
@@ -4395,11 +4395,11 @@
     </row>
     <row r="73" spans="1:14">
       <c r="A73" s="0">
-        <v>50015784</v>
+        <v>50015883</v>
       </c>
       <c r="B73" s="0" t="inlineStr">
         <is>
-          <t>天空</t>
+          <t>A00金华义乌叉车出租电15268650979</t>
         </is>
       </c>
       <c r="C73" s="0" t="inlineStr">
@@ -4424,7 +4424,7 @@
       </c>
       <c r="G73" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:41</t>
+          <t>2026-09-03 23:18:02</t>
         </is>
       </c>
       <c r="H73" s="0" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="I73" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J73" s="0" t="inlineStr">
@@ -4455,11 +4455,11 @@
     </row>
     <row r="74" spans="1:14">
       <c r="A74" s="0">
-        <v>50015778</v>
+        <v>50015882</v>
       </c>
       <c r="B74" s="0" t="inlineStr">
         <is>
-          <t>小龙女</t>
+          <t>建程仓储中心 张川</t>
         </is>
       </c>
       <c r="C74" s="0" t="inlineStr">
@@ -4484,7 +4484,7 @@
       </c>
       <c r="G74" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:21</t>
+          <t>2026-09-03 23:18:02</t>
         </is>
       </c>
       <c r="H74" s="0" t="inlineStr">
@@ -4515,11 +4515,11 @@
     </row>
     <row r="75" spans="1:14">
       <c r="A75" s="0">
-        <v>50015776</v>
+        <v>50015784</v>
       </c>
       <c r="B75" s="0" t="inlineStr">
         <is>
-          <t>桥梁</t>
+          <t>天空</t>
         </is>
       </c>
       <c r="C75" s="0" t="inlineStr">
@@ -4544,7 +4544,7 @@
       </c>
       <c r="G75" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:15</t>
+          <t>2026-09-03 23:10:41</t>
         </is>
       </c>
       <c r="H75" s="0" t="inlineStr">
@@ -4575,11 +4575,11 @@
     </row>
     <row r="76" spans="1:14">
       <c r="A76" s="0">
-        <v>50015775</v>
+        <v>50015778</v>
       </c>
       <c r="B76" s="0" t="inlineStr">
         <is>
-          <t>彩云之南</t>
+          <t>小龙女</t>
         </is>
       </c>
       <c r="C76" s="0" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="G76" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:13</t>
+          <t>2026-09-03 23:10:21</t>
         </is>
       </c>
       <c r="H76" s="0" t="inlineStr">
@@ -4635,11 +4635,11 @@
     </row>
     <row r="77" spans="1:14">
       <c r="A77" s="0">
-        <v>50015774</v>
+        <v>50015776</v>
       </c>
       <c r="B77" s="0" t="inlineStr">
         <is>
-          <t>楊精蓄銳༒</t>
+          <t>桥梁</t>
         </is>
       </c>
       <c r="C77" s="0" t="inlineStr">
@@ -4664,7 +4664,7 @@
       </c>
       <c r="G77" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:11</t>
+          <t>2026-09-03 23:10:15</t>
         </is>
       </c>
       <c r="H77" s="0" t="inlineStr">
@@ -4695,11 +4695,11 @@
     </row>
     <row r="78" spans="1:14">
       <c r="A78" s="0">
-        <v>50015772</v>
+        <v>50015775</v>
       </c>
       <c r="B78" s="0" t="inlineStr">
         <is>
-          <t>不倒翁</t>
+          <t>彩云之南</t>
         </is>
       </c>
       <c r="C78" s="0" t="inlineStr">
@@ -4724,7 +4724,7 @@
       </c>
       <c r="G78" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:07</t>
+          <t>2026-09-03 23:10:13</t>
         </is>
       </c>
       <c r="H78" s="0" t="inlineStr">
@@ -4755,11 +4755,11 @@
     </row>
     <row r="79" spans="1:14">
       <c r="A79" s="0">
-        <v>50015770</v>
+        <v>50015774</v>
       </c>
       <c r="B79" s="0" t="inlineStr">
         <is>
-          <t>一江春水</t>
+          <t>楊精蓄銳༒</t>
         </is>
       </c>
       <c r="C79" s="0" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="G79" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:05</t>
+          <t>2026-09-03 23:10:11</t>
         </is>
       </c>
       <c r="H79" s="0" t="inlineStr">
@@ -4815,11 +4815,11 @@
     </row>
     <row r="80" spans="1:14">
       <c r="A80" s="0">
-        <v>50015767</v>
+        <v>50015772</v>
       </c>
       <c r="B80" s="0" t="inlineStr">
         <is>
-          <t>微笑</t>
+          <t>不倒翁</t>
         </is>
       </c>
       <c r="C80" s="0" t="inlineStr">
@@ -4844,7 +4844,7 @@
       </c>
       <c r="G80" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:10:03</t>
+          <t>2026-09-03 23:10:07</t>
         </is>
       </c>
       <c r="H80" s="0" t="inlineStr">
@@ -4875,11 +4875,11 @@
     </row>
     <row r="81" spans="1:14">
       <c r="A81" s="0">
-        <v>50015763</v>
+        <v>50015770</v>
       </c>
       <c r="B81" s="0" t="inlineStr">
         <is>
-          <t>北斗星</t>
+          <t>一江春水</t>
         </is>
       </c>
       <c r="C81" s="0" t="inlineStr">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="G81" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 23:09:39</t>
+          <t>2026-09-03 23:10:05</t>
         </is>
       </c>
       <c r="H81" s="0" t="inlineStr">
@@ -4935,11 +4935,11 @@
     </row>
     <row r="82" spans="1:14">
       <c r="A82" s="0">
-        <v>49989442</v>
+        <v>50015767</v>
       </c>
       <c r="B82" s="0" t="inlineStr">
         <is>
-          <t>冬梅花儿开王丽君</t>
+          <t>微笑</t>
         </is>
       </c>
       <c r="C82" s="0" t="inlineStr">
@@ -4964,7 +4964,7 @@
       </c>
       <c r="G82" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:43</t>
+          <t>2026-09-03 23:10:03</t>
         </is>
       </c>
       <c r="H82" s="0" t="inlineStr">
@@ -4974,7 +4974,7 @@
       </c>
       <c r="I82" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J82" s="0" t="inlineStr">
@@ -4995,11 +4995,11 @@
     </row>
     <row r="83" spans="1:14">
       <c r="A83" s="0">
-        <v>49989431</v>
+        <v>50015763</v>
       </c>
       <c r="B83" s="0" t="inlineStr">
         <is>
-          <t>风声</t>
+          <t>北斗星</t>
         </is>
       </c>
       <c r="C83" s="0" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="G83" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:25</t>
+          <t>2026-09-03 23:09:39</t>
         </is>
       </c>
       <c r="H83" s="0" t="inlineStr">
@@ -5034,7 +5034,7 @@
       </c>
       <c r="I83" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J83" s="0" t="inlineStr">
@@ -5055,11 +5055,11 @@
     </row>
     <row r="84" spans="1:14">
       <c r="A84" s="0">
-        <v>49989419</v>
+        <v>49989442</v>
       </c>
       <c r="B84" s="0" t="inlineStr">
         <is>
-          <t>胡宾</t>
+          <t>冬梅花儿开王丽君</t>
         </is>
       </c>
       <c r="C84" s="0" t="inlineStr">
@@ -5084,7 +5084,7 @@
       </c>
       <c r="G84" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:13</t>
+          <t>2026-09-03 12:23:43</t>
         </is>
       </c>
       <c r="H84" s="0" t="inlineStr">
@@ -5115,11 +5115,11 @@
     </row>
     <row r="85" spans="1:14">
       <c r="A85" s="0">
-        <v>49989410</v>
+        <v>49989431</v>
       </c>
       <c r="B85" s="0" t="inlineStr">
         <is>
-          <t>永远</t>
+          <t>风声</t>
         </is>
       </c>
       <c r="C85" s="0" t="inlineStr">
@@ -5144,7 +5144,7 @@
       </c>
       <c r="G85" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 12:23:03</t>
+          <t>2026-09-03 12:23:25</t>
         </is>
       </c>
       <c r="H85" s="0" t="inlineStr">
@@ -5175,11 +5175,11 @@
     </row>
     <row r="86" spans="1:14">
       <c r="A86" s="0">
-        <v>49984259</v>
+        <v>49989419</v>
       </c>
       <c r="B86" s="0" t="inlineStr">
         <is>
-          <t>好运包张</t>
+          <t>胡宾</t>
         </is>
       </c>
       <c r="C86" s="0" t="inlineStr">
@@ -5204,7 +5204,7 @@
       </c>
       <c r="G86" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:55:37</t>
+          <t>2026-09-03 12:23:13</t>
         </is>
       </c>
       <c r="H86" s="0" t="inlineStr">
@@ -5214,7 +5214,7 @@
       </c>
       <c r="I86" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J86" s="0" t="inlineStr">
@@ -5235,11 +5235,11 @@
     </row>
     <row r="87" spans="1:14">
       <c r="A87" s="0">
-        <v>49984055</v>
+        <v>49989410</v>
       </c>
       <c r="B87" s="0" t="inlineStr">
         <is>
-          <t>点点星辰</t>
+          <t>永远</t>
         </is>
       </c>
       <c r="C87" s="0" t="inlineStr">
@@ -5264,7 +5264,7 @@
       </c>
       <c r="G87" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:49:33</t>
+          <t>2026-09-03 12:23:03</t>
         </is>
       </c>
       <c r="H87" s="0" t="inlineStr">
@@ -5274,7 +5274,7 @@
       </c>
       <c r="I87" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J87" s="0" t="inlineStr">
@@ -5295,11 +5295,11 @@
     </row>
     <row r="88" spans="1:14">
       <c r="A88" s="0">
-        <v>49983134</v>
+        <v>49984259</v>
       </c>
       <c r="B88" s="0" t="inlineStr">
         <is>
-          <t>Zhangrruzhen张如真</t>
+          <t>好运包张</t>
         </is>
       </c>
       <c r="C88" s="0" t="inlineStr">
@@ -5324,7 +5324,7 @@
       </c>
       <c r="G88" s="0" t="inlineStr">
         <is>
-          <t>2026-09-03 09:25:21</t>
+          <t>2026-09-03 09:55:37</t>
         </is>
       </c>
       <c r="H88" s="0" t="inlineStr">
@@ -5355,11 +5355,11 @@
     </row>
     <row r="89" spans="1:14">
       <c r="A89" s="0">
-        <v>49971209</v>
+        <v>49984055</v>
       </c>
       <c r="B89" s="0" t="inlineStr">
         <is>
-          <t>顺丰顺水</t>
+          <t>点点星辰</t>
         </is>
       </c>
       <c r="C89" s="0" t="inlineStr">
@@ -5384,7 +5384,7 @@
       </c>
       <c r="G89" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:29:41</t>
+          <t>2026-09-03 09:49:33</t>
         </is>
       </c>
       <c r="H89" s="0" t="inlineStr">
@@ -5415,11 +5415,11 @@
     </row>
     <row r="90" spans="1:14">
       <c r="A90" s="0">
-        <v>49970732</v>
+        <v>49983134</v>
       </c>
       <c r="B90" s="0" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Zhangrruzhen张如真</t>
         </is>
       </c>
       <c r="C90" s="0" t="inlineStr">
@@ -5444,7 +5444,7 @@
       </c>
       <c r="G90" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:13:53</t>
+          <t>2026-09-03 09:25:21</t>
         </is>
       </c>
       <c r="H90" s="0" t="inlineStr">
@@ -5454,7 +5454,7 @@
       </c>
       <c r="I90" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J90" s="0" t="inlineStr">
@@ -5475,11 +5475,11 @@
     </row>
     <row r="91" spans="1:14">
       <c r="A91" s="0">
-        <v>49970712</v>
+        <v>49971209</v>
       </c>
       <c r="B91" s="0" t="inlineStr">
         <is>
-          <t>月色琴弦</t>
+          <t>顺丰顺水</t>
         </is>
       </c>
       <c r="C91" s="0" t="inlineStr">
@@ -5504,7 +5504,7 @@
       </c>
       <c r="G91" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:13:07</t>
+          <t>2026-09-02 23:29:41</t>
         </is>
       </c>
       <c r="H91" s="0" t="inlineStr">
@@ -5535,11 +5535,11 @@
     </row>
     <row r="92" spans="1:14">
       <c r="A92" s="0">
-        <v>49970699</v>
+        <v>49970732</v>
       </c>
       <c r="B92" s="0" t="inlineStr">
         <is>
-          <t>铜铃</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="C92" s="0" t="inlineStr">
@@ -5564,7 +5564,7 @@
       </c>
       <c r="G92" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:49</t>
+          <t>2026-09-02 23:13:53</t>
         </is>
       </c>
       <c r="H92" s="0" t="inlineStr">
@@ -5595,11 +5595,11 @@
     </row>
     <row r="93" spans="1:14">
       <c r="A93" s="0">
-        <v>49970698</v>
+        <v>49970712</v>
       </c>
       <c r="B93" s="0" t="inlineStr">
         <is>
-          <t>东风吹</t>
+          <t>月色琴弦</t>
         </is>
       </c>
       <c r="C93" s="0" t="inlineStr">
@@ -5624,7 +5624,7 @@
       </c>
       <c r="G93" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:47</t>
+          <t>2026-09-02 23:13:07</t>
         </is>
       </c>
       <c r="H93" s="0" t="inlineStr">
@@ -5655,11 +5655,11 @@
     </row>
     <row r="94" spans="1:14">
       <c r="A94" s="0">
-        <v>49970683</v>
+        <v>49970699</v>
       </c>
       <c r="B94" s="0" t="inlineStr">
         <is>
-          <t>杨永强</t>
+          <t>铜铃</t>
         </is>
       </c>
       <c r="C94" s="0" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="G94" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:12:17</t>
+          <t>2026-09-02 23:12:49</t>
         </is>
       </c>
       <c r="H94" s="0" t="inlineStr">
@@ -5715,11 +5715,11 @@
     </row>
     <row r="95" spans="1:14">
       <c r="A95" s="0">
-        <v>49970662</v>
+        <v>49970698</v>
       </c>
       <c r="B95" s="0" t="inlineStr">
         <is>
-          <t>盈丰</t>
+          <t>东风吹</t>
         </is>
       </c>
       <c r="C95" s="0" t="inlineStr">
@@ -5744,7 +5744,7 @@
       </c>
       <c r="G95" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:33</t>
+          <t>2026-09-02 23:12:47</t>
         </is>
       </c>
       <c r="H95" s="0" t="inlineStr">
@@ -5775,11 +5775,11 @@
     </row>
     <row r="96" spans="1:14">
       <c r="A96" s="0">
-        <v>49970652</v>
+        <v>49970683</v>
       </c>
       <c r="B96" s="0" t="inlineStr">
         <is>
-          <t>YAN</t>
+          <t>杨永强</t>
         </is>
       </c>
       <c r="C96" s="0" t="inlineStr">
@@ -5804,7 +5804,7 @@
       </c>
       <c r="G96" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:15</t>
+          <t>2026-09-02 23:12:17</t>
         </is>
       </c>
       <c r="H96" s="0" t="inlineStr">
@@ -5835,11 +5835,11 @@
     </row>
     <row r="97" spans="1:14">
       <c r="A97" s="0">
-        <v>49970649</v>
+        <v>49970662</v>
       </c>
       <c r="B97" s="0" t="inlineStr">
         <is>
-          <t>彩虹（宋荷娣）</t>
+          <t>盈丰</t>
         </is>
       </c>
       <c r="C97" s="0" t="inlineStr">
@@ -5864,7 +5864,7 @@
       </c>
       <c r="G97" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:11</t>
+          <t>2026-09-02 23:11:33</t>
         </is>
       </c>
       <c r="H97" s="0" t="inlineStr">
@@ -5895,11 +5895,11 @@
     </row>
     <row r="98" spans="1:14">
       <c r="A98" s="0">
-        <v>49970648</v>
+        <v>49970652</v>
       </c>
       <c r="B98" s="0" t="inlineStr">
         <is>
-          <t>天知心</t>
+          <t>YAN</t>
         </is>
       </c>
       <c r="C98" s="0" t="inlineStr">
@@ -5924,7 +5924,7 @@
       </c>
       <c r="G98" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:11:08</t>
+          <t>2026-09-02 23:11:15</t>
         </is>
       </c>
       <c r="H98" s="0" t="inlineStr">
@@ -5955,11 +5955,11 @@
     </row>
     <row r="99" spans="1:14">
       <c r="A99" s="0">
-        <v>49970643</v>
+        <v>49970649</v>
       </c>
       <c r="B99" s="0" t="inlineStr">
         <is>
-          <t>好运来</t>
+          <t>彩虹（宋荷娣）</t>
         </is>
       </c>
       <c r="C99" s="0" t="inlineStr">
@@ -5984,7 +5984,7 @@
       </c>
       <c r="G99" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 23:10:55</t>
+          <t>2026-09-02 23:11:11</t>
         </is>
       </c>
       <c r="H99" s="0" t="inlineStr">
@@ -6015,11 +6015,11 @@
     </row>
     <row r="100" spans="1:14">
       <c r="A100" s="0">
-        <v>49937566</v>
+        <v>49970648</v>
       </c>
       <c r="B100" s="0" t="inlineStr">
         <is>
-          <t>简单sincerity</t>
+          <t>天知心</t>
         </is>
       </c>
       <c r="C100" s="0" t="inlineStr">
@@ -6044,7 +6044,7 @@
       </c>
       <c r="G100" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 10:10:33</t>
+          <t>2026-09-02 23:11:08</t>
         </is>
       </c>
       <c r="H100" s="0" t="inlineStr">
@@ -6075,11 +6075,11 @@
     </row>
     <row r="101" spans="1:14">
       <c r="A101" s="0">
-        <v>49937187</v>
+        <v>49970643</v>
       </c>
       <c r="B101" s="0" t="inlineStr">
         <is>
-          <t>莲子</t>
+          <t>好运来</t>
         </is>
       </c>
       <c r="C101" s="0" t="inlineStr">
@@ -6104,7 +6104,7 @@
       </c>
       <c r="G101" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:58:56</t>
+          <t>2026-09-02 23:10:55</t>
         </is>
       </c>
       <c r="H101" s="0" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="I101" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J101" s="0" t="inlineStr">
@@ -6135,11 +6135,11 @@
     </row>
     <row r="102" spans="1:14">
       <c r="A102" s="0">
-        <v>49937101</v>
+        <v>49937566</v>
       </c>
       <c r="B102" s="0" t="inlineStr">
         <is>
-          <t>蓉儿</t>
+          <t>简单sincerity</t>
         </is>
       </c>
       <c r="C102" s="0" t="inlineStr">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="G102" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:56:16</t>
+          <t>2026-09-02 10:10:33</t>
         </is>
       </c>
       <c r="H102" s="0" t="inlineStr">
@@ -6195,11 +6195,11 @@
     </row>
     <row r="103" spans="1:14">
       <c r="A103" s="0">
-        <v>49937098</v>
+        <v>49937187</v>
       </c>
       <c r="B103" s="0" t="inlineStr">
         <is>
-          <t>瀚林2368</t>
+          <t>莲子</t>
         </is>
       </c>
       <c r="C103" s="0" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="G103" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:56:15</t>
+          <t>2026-09-02 09:58:56</t>
         </is>
       </c>
       <c r="H103" s="0" t="inlineStr">
@@ -6234,7 +6234,7 @@
       </c>
       <c r="I103" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J103" s="0" t="inlineStr">
@@ -6255,11 +6255,11 @@
     </row>
     <row r="104" spans="1:14">
       <c r="A104" s="0">
-        <v>49937081</v>
+        <v>49937101</v>
       </c>
       <c r="B104" s="0" t="inlineStr">
         <is>
-          <t>🔱 花中之美</t>
+          <t>蓉儿</t>
         </is>
       </c>
       <c r="C104" s="0" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="G104" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:47</t>
+          <t>2026-09-02 09:56:16</t>
         </is>
       </c>
       <c r="H104" s="0" t="inlineStr">
@@ -6315,11 +6315,11 @@
     </row>
     <row r="105" spans="1:14">
       <c r="A105" s="0">
-        <v>49937066</v>
+        <v>49937098</v>
       </c>
       <c r="B105" s="0" t="inlineStr">
         <is>
-          <t>雨情</t>
+          <t>瀚林2368</t>
         </is>
       </c>
       <c r="C105" s="0" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="G105" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:27</t>
+          <t>2026-09-02 09:56:15</t>
         </is>
       </c>
       <c r="H105" s="0" t="inlineStr">
@@ -6375,11 +6375,11 @@
     </row>
     <row r="106" spans="1:14">
       <c r="A106" s="0">
-        <v>49937061</v>
+        <v>49937081</v>
       </c>
       <c r="B106" s="0" t="inlineStr">
         <is>
-          <t>Sunny 🎈瑶</t>
+          <t>🔱 花中之美</t>
         </is>
       </c>
       <c r="C106" s="0" t="inlineStr">
@@ -6404,7 +6404,7 @@
       </c>
       <c r="G106" s="0" t="inlineStr">
         <is>
-          <t>2026-09-02 09:55:23</t>
+          <t>2026-09-02 09:55:47</t>
         </is>
       </c>
       <c r="H106" s="0" t="inlineStr">
@@ -6435,11 +6435,11 @@
     </row>
     <row r="107" spans="1:14">
       <c r="A107" s="0">
-        <v>49887876</v>
+        <v>49937066</v>
       </c>
       <c r="B107" s="0" t="inlineStr">
         <is>
-          <t>鱼靖儿</t>
+          <t>雨情</t>
         </is>
       </c>
       <c r="C107" s="0" t="inlineStr">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="G107" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:23:11</t>
+          <t>2026-09-02 09:55:27</t>
         </is>
       </c>
       <c r="H107" s="0" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="I107" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J107" s="0" t="inlineStr">
@@ -6495,11 +6495,11 @@
     </row>
     <row r="108" spans="1:14">
       <c r="A108" s="0">
-        <v>49887478</v>
+        <v>49937061</v>
       </c>
       <c r="B108" s="0" t="inlineStr">
         <is>
-          <t>风调雨顺</t>
+          <t>Sunny 🎈瑶</t>
         </is>
       </c>
       <c r="C108" s="0" t="inlineStr">
@@ -6524,7 +6524,7 @@
       </c>
       <c r="G108" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:10:17</t>
+          <t>2026-09-02 09:55:23</t>
         </is>
       </c>
       <c r="H108" s="0" t="inlineStr">
@@ -6555,11 +6555,11 @@
     </row>
     <row r="109" spans="1:14">
       <c r="A109" s="0">
-        <v>49887447</v>
+        <v>49887876</v>
       </c>
       <c r="B109" s="0" t="inlineStr">
         <is>
-          <t>中国艺人</t>
+          <t>鱼靖儿</t>
         </is>
       </c>
       <c r="C109" s="0" t="inlineStr">
@@ -6584,7 +6584,7 @@
       </c>
       <c r="G109" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:44</t>
+          <t>2026-08-31 23:23:11</t>
         </is>
       </c>
       <c r="H109" s="0" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="I109" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J109" s="0" t="inlineStr">
@@ -6615,11 +6615,11 @@
     </row>
     <row r="110" spans="1:14">
       <c r="A110" s="0">
-        <v>49887439</v>
+        <v>49887478</v>
       </c>
       <c r="B110" s="0" t="inlineStr">
         <is>
-          <t>黄晓玲</t>
+          <t>风调雨顺</t>
         </is>
       </c>
       <c r="C110" s="0" t="inlineStr">
@@ -6644,7 +6644,7 @@
       </c>
       <c r="G110" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:17</t>
+          <t>2026-08-31 23:10:17</t>
         </is>
       </c>
       <c r="H110" s="0" t="inlineStr">
@@ -6675,11 +6675,11 @@
     </row>
     <row r="111" spans="1:14">
       <c r="A111" s="0">
-        <v>49887437</v>
+        <v>49887447</v>
       </c>
       <c r="B111" s="0" t="inlineStr">
         <is>
-          <t>随缘</t>
+          <t>中国艺人</t>
         </is>
       </c>
       <c r="C111" s="0" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="G111" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:08:07</t>
+          <t>2026-08-31 23:08:44</t>
         </is>
       </c>
       <c r="H111" s="0" t="inlineStr">
@@ -6735,11 +6735,11 @@
     </row>
     <row r="112" spans="1:14">
       <c r="A112" s="0">
-        <v>49887416</v>
+        <v>49887439</v>
       </c>
       <c r="B112" s="0" t="inlineStr">
         <is>
-          <t>刘秋红</t>
+          <t>黄晓玲</t>
         </is>
       </c>
       <c r="C112" s="0" t="inlineStr">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="G112" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:31</t>
+          <t>2026-08-31 23:08:17</t>
         </is>
       </c>
       <c r="H112" s="0" t="inlineStr">
@@ -6795,11 +6795,11 @@
     </row>
     <row r="113" spans="1:14">
       <c r="A113" s="0">
-        <v>49887403</v>
+        <v>49887437</v>
       </c>
       <c r="B113" s="0" t="inlineStr">
         <is>
-          <t>Mr.</t>
+          <t>随缘</t>
         </is>
       </c>
       <c r="C113" s="0" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="G113" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:05</t>
+          <t>2026-08-31 23:08:07</t>
         </is>
       </c>
       <c r="H113" s="0" t="inlineStr">
@@ -6855,11 +6855,11 @@
     </row>
     <row r="114" spans="1:14">
       <c r="A114" s="0">
-        <v>49887401</v>
+        <v>49887416</v>
       </c>
       <c r="B114" s="0" t="inlineStr">
         <is>
-          <t>万事如意</t>
+          <t>刘秋红</t>
         </is>
       </c>
       <c r="C114" s="0" t="inlineStr">
@@ -6884,7 +6884,7 @@
       </c>
       <c r="G114" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:03</t>
+          <t>2026-08-31 23:07:31</t>
         </is>
       </c>
       <c r="H114" s="0" t="inlineStr">
@@ -6915,11 +6915,11 @@
     </row>
     <row r="115" spans="1:14">
       <c r="A115" s="0">
-        <v>49887400</v>
+        <v>49887403</v>
       </c>
       <c r="B115" s="0" t="inlineStr">
         <is>
-          <t>💋诺墨</t>
+          <t>Mr.</t>
         </is>
       </c>
       <c r="C115" s="0" t="inlineStr">
@@ -6944,7 +6944,7 @@
       </c>
       <c r="G115" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:07:01</t>
+          <t>2026-08-31 23:07:05</t>
         </is>
       </c>
       <c r="H115" s="0" t="inlineStr">
@@ -6975,11 +6975,11 @@
     </row>
     <row r="116" spans="1:14">
       <c r="A116" s="0">
-        <v>49887399</v>
+        <v>49887401</v>
       </c>
       <c r="B116" s="0" t="inlineStr">
         <is>
-          <t>听风</t>
+          <t>万事如意</t>
         </is>
       </c>
       <c r="C116" s="0" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="G116" s="0" t="inlineStr">
         <is>
-          <t>2026-08-31 23:06:59</t>
+          <t>2026-08-31 23:07:03</t>
         </is>
       </c>
       <c r="H116" s="0" t="inlineStr">
@@ -7035,11 +7035,11 @@
     </row>
     <row r="117" spans="1:14">
       <c r="A117" s="0">
-        <v>49845584</v>
+        <v>49887400</v>
       </c>
       <c r="B117" s="0" t="inlineStr">
         <is>
-          <t>彭汉平13024282926</t>
+          <t>💋诺墨</t>
         </is>
       </c>
       <c r="C117" s="0" t="inlineStr">
@@ -7064,7 +7064,7 @@
       </c>
       <c r="G117" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:18:55</t>
+          <t>2026-08-31 23:07:01</t>
         </is>
       </c>
       <c r="H117" s="0" t="inlineStr">
@@ -7095,11 +7095,11 @@
     </row>
     <row r="118" spans="1:14">
       <c r="A118" s="0">
-        <v>49845487</v>
+        <v>49887399</v>
       </c>
       <c r="B118" s="0" t="inlineStr">
         <is>
-          <t>Z国华</t>
+          <t>听风</t>
         </is>
       </c>
       <c r="C118" s="0" t="inlineStr">
@@ -7124,7 +7124,7 @@
       </c>
       <c r="G118" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:15:49</t>
+          <t>2026-08-31 23:06:59</t>
         </is>
       </c>
       <c r="H118" s="0" t="inlineStr">
@@ -7134,7 +7134,7 @@
       </c>
       <c r="I118" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J118" s="0" t="inlineStr">
@@ -7155,11 +7155,11 @@
     </row>
     <row r="119" spans="1:14">
       <c r="A119" s="0">
-        <v>49845407</v>
+        <v>49845584</v>
       </c>
       <c r="B119" s="0" t="inlineStr">
         <is>
-          <t>月亮🌛</t>
+          <t>彭汉平13024282926</t>
         </is>
       </c>
       <c r="C119" s="0" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="G119" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:12:33</t>
+          <t>2026-08-30 23:18:55</t>
         </is>
       </c>
       <c r="H119" s="0" t="inlineStr">
@@ -7215,11 +7215,11 @@
     </row>
     <row r="120" spans="1:14">
       <c r="A120" s="0">
-        <v>49845398</v>
+        <v>49845487</v>
       </c>
       <c r="B120" s="0" t="inlineStr">
         <is>
-          <t>老树</t>
+          <t>Z国华</t>
         </is>
       </c>
       <c r="C120" s="0" t="inlineStr">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="G120" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:12:03</t>
+          <t>2026-08-30 23:15:49</t>
         </is>
       </c>
       <c r="H120" s="0" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="I120" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J120" s="0" t="inlineStr">
@@ -7275,11 +7275,11 @@
     </row>
     <row r="121" spans="1:14">
       <c r="A121" s="0">
-        <v>49845391</v>
+        <v>49845407</v>
       </c>
       <c r="B121" s="0" t="inlineStr">
         <is>
-          <t>八哥</t>
+          <t>月亮🌛</t>
         </is>
       </c>
       <c r="C121" s="0" t="inlineStr">
@@ -7304,7 +7304,7 @@
       </c>
       <c r="G121" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:45</t>
+          <t>2026-08-30 23:12:33</t>
         </is>
       </c>
       <c r="H121" s="0" t="inlineStr">
@@ -7335,11 +7335,11 @@
     </row>
     <row r="122" spans="1:14">
       <c r="A122" s="0">
-        <v>49845380</v>
+        <v>49845398</v>
       </c>
       <c r="B122" s="0" t="inlineStr">
         <is>
-          <t>铲车主出租15352562068</t>
+          <t>老树</t>
         </is>
       </c>
       <c r="C122" s="0" t="inlineStr">
@@ -7364,7 +7364,7 @@
       </c>
       <c r="G122" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:29</t>
+          <t>2026-08-30 23:12:03</t>
         </is>
       </c>
       <c r="H122" s="0" t="inlineStr">
@@ -7395,11 +7395,11 @@
     </row>
     <row r="123" spans="1:14">
       <c r="A123" s="0">
-        <v>49845376</v>
+        <v>49845391</v>
       </c>
       <c r="B123" s="0" t="inlineStr">
         <is>
-          <t>刘萍</t>
+          <t>八哥</t>
         </is>
       </c>
       <c r="C123" s="0" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="G123" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:15</t>
+          <t>2026-08-30 23:11:45</t>
         </is>
       </c>
       <c r="H123" s="0" t="inlineStr">
@@ -7455,11 +7455,11 @@
     </row>
     <row r="124" spans="1:14">
       <c r="A124" s="0">
-        <v>49845374</v>
+        <v>49845380</v>
       </c>
       <c r="B124" s="0" t="inlineStr">
         <is>
-          <t>空谷幽兰</t>
+          <t>铲车主出租15352562068</t>
         </is>
       </c>
       <c r="C124" s="0" t="inlineStr">
@@ -7484,7 +7484,7 @@
       </c>
       <c r="G124" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:07</t>
+          <t>2026-08-30 23:11:29</t>
         </is>
       </c>
       <c r="H124" s="0" t="inlineStr">
@@ -7515,11 +7515,11 @@
     </row>
     <row r="125" spans="1:14">
       <c r="A125" s="0">
-        <v>49845373</v>
+        <v>49845376</v>
       </c>
       <c r="B125" s="0" t="inlineStr">
         <is>
-          <t>泽浩羊</t>
+          <t>刘萍</t>
         </is>
       </c>
       <c r="C125" s="0" t="inlineStr">
@@ -7544,7 +7544,7 @@
       </c>
       <c r="G125" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:11:05</t>
+          <t>2026-08-30 23:11:15</t>
         </is>
       </c>
       <c r="H125" s="0" t="inlineStr">
@@ -7575,11 +7575,11 @@
     </row>
     <row r="126" spans="1:14">
       <c r="A126" s="0">
-        <v>49845367</v>
+        <v>49845374</v>
       </c>
       <c r="B126" s="0" t="inlineStr">
         <is>
-          <t>峰回路转</t>
+          <t>空谷幽兰</t>
         </is>
       </c>
       <c r="C126" s="0" t="inlineStr">
@@ -7604,7 +7604,7 @@
       </c>
       <c r="G126" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:55</t>
+          <t>2026-08-30 23:11:07</t>
         </is>
       </c>
       <c r="H126" s="0" t="inlineStr">
@@ -7635,11 +7635,11 @@
     </row>
     <row r="127" spans="1:14">
       <c r="A127" s="0">
-        <v>49845366</v>
+        <v>49845373</v>
       </c>
       <c r="B127" s="0" t="inlineStr">
         <is>
-          <t>超儿</t>
+          <t>泽浩羊</t>
         </is>
       </c>
       <c r="C127" s="0" t="inlineStr">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="G127" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:51</t>
+          <t>2026-08-30 23:11:05</t>
         </is>
       </c>
       <c r="H127" s="0" t="inlineStr">
@@ -7695,11 +7695,11 @@
     </row>
     <row r="128" spans="1:14">
       <c r="A128" s="0">
-        <v>49845365</v>
+        <v>49845367</v>
       </c>
       <c r="B128" s="0" t="inlineStr">
         <is>
-          <t>传</t>
+          <t>峰回路转</t>
         </is>
       </c>
       <c r="C128" s="0" t="inlineStr">
@@ -7724,7 +7724,7 @@
       </c>
       <c r="G128" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:49</t>
+          <t>2026-08-30 23:10:55</t>
         </is>
       </c>
       <c r="H128" s="0" t="inlineStr">
@@ -7755,11 +7755,11 @@
     </row>
     <row r="129" spans="1:14">
       <c r="A129" s="0">
-        <v>49845360</v>
+        <v>49845366</v>
       </c>
       <c r="B129" s="0" t="inlineStr">
         <is>
-          <t>悟歌</t>
+          <t>超儿</t>
         </is>
       </c>
       <c r="C129" s="0" t="inlineStr">
@@ -7784,7 +7784,7 @@
       </c>
       <c r="G129" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:43</t>
+          <t>2026-08-30 23:10:51</t>
         </is>
       </c>
       <c r="H129" s="0" t="inlineStr">
@@ -7815,11 +7815,11 @@
     </row>
     <row r="130" spans="1:14">
       <c r="A130" s="0">
-        <v>49845342</v>
+        <v>49845365</v>
       </c>
       <c r="B130" s="0" t="inlineStr">
         <is>
-          <t>丽丽</t>
+          <t>传</t>
         </is>
       </c>
       <c r="C130" s="0" t="inlineStr">
@@ -7844,7 +7844,7 @@
       </c>
       <c r="G130" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 23:10:15</t>
+          <t>2026-08-30 23:10:49</t>
         </is>
       </c>
       <c r="H130" s="0" t="inlineStr">
@@ -7875,11 +7875,11 @@
     </row>
     <row r="131" spans="1:14">
       <c r="A131" s="0">
-        <v>49826011</v>
+        <v>49845360</v>
       </c>
       <c r="B131" s="0" t="inlineStr">
         <is>
-          <t>王前卫</t>
+          <t>悟歌</t>
         </is>
       </c>
       <c r="C131" s="0" t="inlineStr">
@@ -7904,7 +7904,7 @@
       </c>
       <c r="G131" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:57:27</t>
+          <t>2026-08-30 23:10:43</t>
         </is>
       </c>
       <c r="H131" s="0" t="inlineStr">
@@ -7935,11 +7935,11 @@
     </row>
     <row r="132" spans="1:14">
       <c r="A132" s="0">
-        <v>49825720</v>
+        <v>49845342</v>
       </c>
       <c r="B132" s="0" t="inlineStr">
         <is>
-          <t>老A</t>
+          <t>丽丽</t>
         </is>
       </c>
       <c r="C132" s="0" t="inlineStr">
@@ -7964,7 +7964,7 @@
       </c>
       <c r="G132" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:46:02</t>
+          <t>2026-08-30 23:10:15</t>
         </is>
       </c>
       <c r="H132" s="0" t="inlineStr">
@@ -7995,11 +7995,11 @@
     </row>
     <row r="133" spans="1:14">
       <c r="A133" s="0">
-        <v>49825676</v>
+        <v>49826011</v>
       </c>
       <c r="B133" s="0" t="inlineStr">
         <is>
-          <t>蓝天</t>
+          <t>王前卫</t>
         </is>
       </c>
       <c r="C133" s="0" t="inlineStr">
@@ -8024,7 +8024,7 @@
       </c>
       <c r="G133" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:44:05</t>
+          <t>2026-08-30 12:57:27</t>
         </is>
       </c>
       <c r="H133" s="0" t="inlineStr">
@@ -8055,11 +8055,11 @@
     </row>
     <row r="134" spans="1:14">
       <c r="A134" s="0">
-        <v>49825650</v>
+        <v>49825720</v>
       </c>
       <c r="B134" s="0" t="inlineStr">
         <is>
-          <t>爱芳</t>
+          <t>老A</t>
         </is>
       </c>
       <c r="C134" s="0" t="inlineStr">
@@ -8084,7 +8084,7 @@
       </c>
       <c r="G134" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:43:11</t>
+          <t>2026-08-30 12:46:02</t>
         </is>
       </c>
       <c r="H134" s="0" t="inlineStr">
@@ -8115,11 +8115,11 @@
     </row>
     <row r="135" spans="1:14">
       <c r="A135" s="0">
-        <v>49825642</v>
+        <v>49825676</v>
       </c>
       <c r="B135" s="0" t="inlineStr">
         <is>
-          <t>银杏树</t>
+          <t>蓝天</t>
         </is>
       </c>
       <c r="C135" s="0" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="G135" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:55</t>
+          <t>2026-08-30 12:44:05</t>
         </is>
       </c>
       <c r="H135" s="0" t="inlineStr">
@@ -8175,11 +8175,11 @@
     </row>
     <row r="136" spans="1:14">
       <c r="A136" s="0">
-        <v>49825640</v>
+        <v>49825650</v>
       </c>
       <c r="B136" s="0" t="inlineStr">
         <is>
-          <t>遵命有福（杨凤）</t>
+          <t>爱芳</t>
         </is>
       </c>
       <c r="C136" s="0" t="inlineStr">
@@ -8204,7 +8204,7 @@
       </c>
       <c r="G136" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:49</t>
+          <t>2026-08-30 12:43:11</t>
         </is>
       </c>
       <c r="H136" s="0" t="inlineStr">
@@ -8235,11 +8235,11 @@
     </row>
     <row r="137" spans="1:14">
       <c r="A137" s="0">
-        <v>49825639</v>
+        <v>49825642</v>
       </c>
       <c r="B137" s="0" t="inlineStr">
         <is>
-          <t>申华</t>
+          <t>银杏树</t>
         </is>
       </c>
       <c r="C137" s="0" t="inlineStr">
@@ -8264,7 +8264,7 @@
       </c>
       <c r="G137" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:49</t>
+          <t>2026-08-30 12:42:55</t>
         </is>
       </c>
       <c r="H137" s="0" t="inlineStr">
@@ -8295,11 +8295,11 @@
     </row>
     <row r="138" spans="1:14">
       <c r="A138" s="0">
-        <v>49825637</v>
+        <v>49825640</v>
       </c>
       <c r="B138" s="0" t="inlineStr">
         <is>
-          <t>陈月焓</t>
+          <t>遵命有福（杨凤）</t>
         </is>
       </c>
       <c r="C138" s="0" t="inlineStr">
@@ -8324,7 +8324,7 @@
       </c>
       <c r="G138" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:47</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H138" s="0" t="inlineStr">
@@ -8355,11 +8355,11 @@
     </row>
     <row r="139" spans="1:14">
       <c r="A139" s="0">
-        <v>49825635</v>
+        <v>49825639</v>
       </c>
       <c r="B139" s="0" t="inlineStr">
         <is>
-          <t>小镇生活&amp;&amp;杜震</t>
+          <t>申华</t>
         </is>
       </c>
       <c r="C139" s="0" t="inlineStr">
@@ -8384,7 +8384,7 @@
       </c>
       <c r="G139" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:43</t>
+          <t>2026-08-30 12:42:49</t>
         </is>
       </c>
       <c r="H139" s="0" t="inlineStr">
@@ -8415,11 +8415,11 @@
     </row>
     <row r="140" spans="1:14">
       <c r="A140" s="0">
-        <v>49825628</v>
+        <v>49825637</v>
       </c>
       <c r="B140" s="0" t="inlineStr">
         <is>
-          <t>Taᴗaoᥫᩣ</t>
+          <t>陈月焓</t>
         </is>
       </c>
       <c r="C140" s="0" t="inlineStr">
@@ -8444,7 +8444,7 @@
       </c>
       <c r="G140" s="0" t="inlineStr">
         <is>
-          <t>2026-08-30 12:42:35</t>
+          <t>2026-08-30 12:42:47</t>
         </is>
       </c>
       <c r="H140" s="0" t="inlineStr">
@@ -8475,11 +8475,11 @@
     </row>
     <row r="141" spans="1:14">
       <c r="A141" s="0">
-        <v>49782066</v>
+        <v>49825635</v>
       </c>
       <c r="B141" s="0" t="inlineStr">
         <is>
-          <t>前程似锦</t>
+          <t>小镇生活&amp;&amp;杜震</t>
         </is>
       </c>
       <c r="C141" s="0" t="inlineStr">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="G141" s="0" t="inlineStr">
         <is>
-          <t>2026-08-29 09:07:29</t>
+          <t>2026-08-30 12:42:43</t>
         </is>
       </c>
       <c r="H141" s="0" t="inlineStr">
@@ -8514,7 +8514,7 @@
       </c>
       <c r="I141" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J141" s="0" t="inlineStr">
@@ -8535,11 +8535,11 @@
     </row>
     <row r="142" spans="1:14">
       <c r="A142" s="0">
-        <v>49771027</v>
+        <v>49825628</v>
       </c>
       <c r="B142" s="0" t="inlineStr">
         <is>
-          <t>非比</t>
+          <t>Taᴗaoᥫᩣ</t>
         </is>
       </c>
       <c r="C142" s="0" t="inlineStr">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="G142" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 23:30:09</t>
+          <t>2026-08-30 12:42:35</t>
         </is>
       </c>
       <c r="H142" s="0" t="inlineStr">
@@ -8574,7 +8574,7 @@
       </c>
       <c r="I142" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J142" s="0" t="inlineStr">
@@ -8595,11 +8595,11 @@
     </row>
     <row r="143" spans="1:14">
       <c r="A143" s="0">
-        <v>49673360</v>
+        <v>49782066</v>
       </c>
       <c r="B143" s="0" t="inlineStr">
         <is>
-          <t>德行天下</t>
+          <t>前程似锦</t>
         </is>
       </c>
       <c r="C143" s="0" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="G143" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:19:03</t>
+          <t>2026-08-29 09:07:29</t>
         </is>
       </c>
       <c r="H143" s="0" t="inlineStr">
@@ -8634,7 +8634,7 @@
       </c>
       <c r="I143" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J143" s="0" t="inlineStr">
@@ -8655,11 +8655,11 @@
     </row>
     <row r="144" spans="1:14">
       <c r="A144" s="0">
-        <v>49673352</v>
+        <v>49771027</v>
       </c>
       <c r="B144" s="0" t="inlineStr">
         <is>
-          <t>余盛将至2026</t>
+          <t>非比</t>
         </is>
       </c>
       <c r="C144" s="0" t="inlineStr">
@@ -8684,7 +8684,7 @@
       </c>
       <c r="G144" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:49</t>
+          <t>2026-08-28 23:30:09</t>
         </is>
       </c>
       <c r="H144" s="0" t="inlineStr">
@@ -8694,7 +8694,7 @@
       </c>
       <c r="I144" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音02</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J144" s="0" t="inlineStr">
@@ -8715,11 +8715,11 @@
     </row>
     <row r="145" spans="1:14">
       <c r="A145" s="0">
-        <v>49673350</v>
+        <v>49673360</v>
       </c>
       <c r="B145" s="0" t="inlineStr">
         <is>
-          <t>山居客</t>
+          <t>德行天下</t>
         </is>
       </c>
       <c r="C145" s="0" t="inlineStr">
@@ -8744,7 +8744,7 @@
       </c>
       <c r="G145" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:47</t>
+          <t>2026-08-26 12:19:03</t>
         </is>
       </c>
       <c r="H145" s="0" t="inlineStr">
@@ -8775,11 +8775,11 @@
     </row>
     <row r="146" spans="1:14">
       <c r="A146" s="0">
-        <v>49673349</v>
+        <v>49673352</v>
       </c>
       <c r="B146" s="0" t="inlineStr">
         <is>
-          <t>白云</t>
+          <t>余盛将至2026</t>
         </is>
       </c>
       <c r="C146" s="0" t="inlineStr">
@@ -8804,7 +8804,7 @@
       </c>
       <c r="G146" s="0" t="inlineStr">
         <is>
-          <t>2026-08-26 12:18:45</t>
+          <t>2026-08-26 12:18:49</t>
         </is>
       </c>
       <c r="H146" s="0" t="inlineStr">
@@ -8835,11 +8835,11 @@
     </row>
     <row r="147" spans="1:14">
       <c r="A147" s="0">
-        <v>49646935</v>
+        <v>49673350</v>
       </c>
       <c r="B147" s="0" t="inlineStr">
         <is>
-          <t>马跃荣</t>
+          <t>山居客</t>
         </is>
       </c>
       <c r="C147" s="0" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="G147" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:59</t>
+          <t>2026-08-26 12:18:47</t>
         </is>
       </c>
       <c r="H147" s="0" t="inlineStr">
@@ -8895,11 +8895,11 @@
     </row>
     <row r="148" spans="1:14">
       <c r="A148" s="0">
-        <v>49646933</v>
+        <v>49673349</v>
       </c>
       <c r="B148" s="0" t="inlineStr">
         <is>
-          <t>@吴</t>
+          <t>白云</t>
         </is>
       </c>
       <c r="C148" s="0" t="inlineStr">
@@ -8924,7 +8924,7 @@
       </c>
       <c r="G148" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:15:56</t>
+          <t>2026-08-26 12:18:45</t>
         </is>
       </c>
       <c r="H148" s="0" t="inlineStr">
@@ -8955,11 +8955,11 @@
     </row>
     <row r="149" spans="1:14">
       <c r="A149" s="0">
-        <v>49646901</v>
+        <v>49646935</v>
       </c>
       <c r="B149" s="0" t="inlineStr">
         <is>
-          <t>龙安：富华／</t>
+          <t>马跃荣</t>
         </is>
       </c>
       <c r="C149" s="0" t="inlineStr">
@@ -8984,7 +8984,7 @@
       </c>
       <c r="G149" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:14:28</t>
+          <t>2026-08-25 18:15:59</t>
         </is>
       </c>
       <c r="H149" s="0" t="inlineStr">
@@ -9015,11 +9015,11 @@
     </row>
     <row r="150" spans="1:14">
       <c r="A150" s="0">
-        <v>49646876</v>
+        <v>49646933</v>
       </c>
       <c r="B150" s="0" t="inlineStr">
         <is>
-          <t>冬日暖阳🌻</t>
+          <t>@吴</t>
         </is>
       </c>
       <c r="C150" s="0" t="inlineStr">
@@ -9044,7 +9044,7 @@
       </c>
       <c r="G150" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:37</t>
+          <t>2026-08-25 18:15:56</t>
         </is>
       </c>
       <c r="H150" s="0" t="inlineStr">
@@ -9075,11 +9075,11 @@
     </row>
     <row r="151" spans="1:14">
       <c r="A151" s="0">
-        <v>49646867</v>
+        <v>49646901</v>
       </c>
       <c r="B151" s="0" t="inlineStr">
         <is>
-          <t>寒雨</t>
+          <t>龙安：富华／</t>
         </is>
       </c>
       <c r="C151" s="0" t="inlineStr">
@@ -9104,7 +9104,7 @@
       </c>
       <c r="G151" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 18:13:15</t>
+          <t>2026-08-25 18:14:28</t>
         </is>
       </c>
       <c r="H151" s="0" t="inlineStr">
@@ -9135,11 +9135,11 @@
     </row>
     <row r="152" spans="1:14">
       <c r="A152" s="0">
-        <v>49636232</v>
+        <v>49646876</v>
       </c>
       <c r="B152" s="0" t="inlineStr">
         <is>
-          <t>平安</t>
+          <t>冬日暖阳🌻</t>
         </is>
       </c>
       <c r="C152" s="0" t="inlineStr">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="G152" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:20:15</t>
+          <t>2026-08-25 18:13:37</t>
         </is>
       </c>
       <c r="H152" s="0" t="inlineStr">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="I152" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J152" s="0" t="inlineStr">
@@ -9195,11 +9195,11 @@
     </row>
     <row r="153" spans="1:14">
       <c r="A153" s="0">
-        <v>49636184</v>
+        <v>49646867</v>
       </c>
       <c r="B153" s="0" t="inlineStr">
         <is>
-          <t>古道西风</t>
+          <t>寒雨</t>
         </is>
       </c>
       <c r="C153" s="0" t="inlineStr">
@@ -9224,7 +9224,7 @@
       </c>
       <c r="G153" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:55</t>
+          <t>2026-08-25 18:13:15</t>
         </is>
       </c>
       <c r="H153" s="0" t="inlineStr">
@@ -9234,7 +9234,7 @@
       </c>
       <c r="I153" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-抖音02</t>
         </is>
       </c>
       <c r="J153" s="0" t="inlineStr">
@@ -9255,11 +9255,11 @@
     </row>
     <row r="154" spans="1:14">
       <c r="A154" s="0">
-        <v>49636170</v>
+        <v>49636232</v>
       </c>
       <c r="B154" s="0" t="inlineStr">
         <is>
-          <t>周海龙</t>
+          <t>平安</t>
         </is>
       </c>
       <c r="C154" s="0" t="inlineStr">
@@ -9284,7 +9284,7 @@
       </c>
       <c r="G154" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:33</t>
+          <t>2026-08-25 13:20:15</t>
         </is>
       </c>
       <c r="H154" s="0" t="inlineStr">
@@ -9294,7 +9294,7 @@
       </c>
       <c r="I154" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J154" s="0" t="inlineStr">
@@ -9315,11 +9315,11 @@
     </row>
     <row r="155" spans="1:14">
       <c r="A155" s="0">
-        <v>49636157</v>
+        <v>49636184</v>
       </c>
       <c r="B155" s="0" t="inlineStr">
         <is>
-          <t>锦妍</t>
+          <t>古道西风</t>
         </is>
       </c>
       <c r="C155" s="0" t="inlineStr">
@@ -9344,7 +9344,7 @@
       </c>
       <c r="G155" s="0" t="inlineStr">
         <is>
-          <t>2026-08-25 13:18:07</t>
+          <t>2026-08-25 13:18:55</t>
         </is>
       </c>
       <c r="H155" s="0" t="inlineStr">
@@ -9375,11 +9375,11 @@
     </row>
     <row r="156" spans="1:14">
       <c r="A156" s="0">
-        <v>49593974</v>
+        <v>49636170</v>
       </c>
       <c r="B156" s="0" t="inlineStr">
         <is>
-          <t>兰兰</t>
+          <t>周海龙</t>
         </is>
       </c>
       <c r="C156" s="0" t="inlineStr">
@@ -9404,7 +9404,7 @@
       </c>
       <c r="G156" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:59:53</t>
+          <t>2026-08-25 13:18:33</t>
         </is>
       </c>
       <c r="H156" s="0" t="inlineStr">
@@ -9414,7 +9414,7 @@
       </c>
       <c r="I156" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J156" s="0" t="inlineStr">
@@ -9435,11 +9435,11 @@
     </row>
     <row r="157" spans="1:14">
       <c r="A157" s="0">
-        <v>49593671</v>
+        <v>49636157</v>
       </c>
       <c r="B157" s="0" t="inlineStr">
         <is>
-          <t>准备1号</t>
+          <t>锦妍</t>
         </is>
       </c>
       <c r="C157" s="0" t="inlineStr">
@@ -9464,7 +9464,7 @@
       </c>
       <c r="G157" s="0" t="inlineStr">
         <is>
-          <t>2026-08-24 12:49:27</t>
+          <t>2026-08-25 13:18:07</t>
         </is>
       </c>
       <c r="H157" s="0" t="inlineStr">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="I157" s="0" t="inlineStr">
         <is>
-          <t>黄老师-视频号01</t>
+          <t>黄老师-抖音01</t>
         </is>
       </c>
       <c r="J157" s="0" t="inlineStr">
@@ -9495,11 +9495,11 @@
     </row>
     <row r="158" spans="1:14">
       <c r="A158" s="0">
-        <v>49535916</v>
+        <v>49593974</v>
       </c>
       <c r="B158" s="0" t="inlineStr">
         <is>
-          <t>真诚</t>
+          <t>兰兰</t>
         </is>
       </c>
       <c r="C158" s="0" t="inlineStr">
@@ -9524,7 +9524,7 @@
       </c>
       <c r="G158" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:46:23</t>
+          <t>2026-08-24 12:59:53</t>
         </is>
       </c>
       <c r="H158" s="0" t="inlineStr">
@@ -9555,11 +9555,11 @@
     </row>
     <row r="159" spans="1:14">
       <c r="A159" s="0">
-        <v>49535653</v>
+        <v>49593671</v>
       </c>
       <c r="B159" s="0" t="inlineStr">
         <is>
-          <t>如意家电13368134456维修</t>
+          <t>准备1号</t>
         </is>
       </c>
       <c r="C159" s="0" t="inlineStr">
@@ -9584,7 +9584,7 @@
       </c>
       <c r="G159" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:28:25</t>
+          <t>2026-08-24 12:49:27</t>
         </is>
       </c>
       <c r="H159" s="0" t="inlineStr">
@@ -9615,11 +9615,11 @@
     </row>
     <row r="160" spans="1:14">
       <c r="A160" s="0">
-        <v>49535650</v>
+        <v>49535916</v>
       </c>
       <c r="B160" s="0" t="inlineStr">
         <is>
-          <t>莺莺</t>
+          <t>真诚</t>
         </is>
       </c>
       <c r="C160" s="0" t="inlineStr">
@@ -9644,7 +9644,7 @@
       </c>
       <c r="G160" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 23:27:55</t>
+          <t>2026-08-22 23:46:23</t>
         </is>
       </c>
       <c r="H160" s="0" t="inlineStr">
@@ -9670,21 +9670,16 @@
       <c r="L160" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N160" s="0" t="inlineStr">
-        <is>
-          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="161" spans="1:14">
       <c r="A161" s="0">
-        <v>49508265</v>
+        <v>49535653</v>
       </c>
       <c r="B161" s="0" t="inlineStr">
         <is>
-          <t>爱猫🐱 咪</t>
+          <t>如意家电13368134456维修</t>
         </is>
       </c>
       <c r="C161" s="0" t="inlineStr">
@@ -9709,7 +9704,7 @@
       </c>
       <c r="G161" s="0" t="inlineStr">
         <is>
-          <t>2026-08-22 09:53:41</t>
+          <t>2026-08-22 23:28:25</t>
         </is>
       </c>
       <c r="H161" s="0" t="inlineStr">
@@ -9740,11 +9735,11 @@
     </row>
     <row r="162" spans="1:14">
       <c r="A162" s="0">
-        <v>49493414</v>
+        <v>49535650</v>
       </c>
       <c r="B162" s="0" t="inlineStr">
         <is>
-          <t>惠平</t>
+          <t>莺莺</t>
         </is>
       </c>
       <c r="C162" s="0" t="inlineStr">
@@ -9769,7 +9764,7 @@
       </c>
       <c r="G162" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:53:02</t>
+          <t>2026-08-22 23:27:55</t>
         </is>
       </c>
       <c r="H162" s="0" t="inlineStr">
@@ -9795,16 +9790,21 @@
       <c r="L162" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N162" s="0" t="inlineStr">
+        <is>
+          <t>黄浦</t>
         </is>
       </c>
     </row>
     <row r="163" spans="1:14">
       <c r="A163" s="0">
-        <v>49493126</v>
+        <v>49508265</v>
       </c>
       <c r="B163" s="0" t="inlineStr">
         <is>
-          <t>刘盼昭</t>
+          <t>爱猫🐱 咪</t>
         </is>
       </c>
       <c r="C163" s="0" t="inlineStr">
@@ -9829,7 +9829,7 @@
       </c>
       <c r="G163" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:44:53</t>
+          <t>2026-08-22 09:53:41</t>
         </is>
       </c>
       <c r="H163" s="0" t="inlineStr">
@@ -9860,11 +9860,11 @@
     </row>
     <row r="164" spans="1:14">
       <c r="A164" s="0">
-        <v>49492499</v>
+        <v>49493414</v>
       </c>
       <c r="B164" s="0" t="inlineStr">
         <is>
-          <t>红霞</t>
+          <t>惠平</t>
         </is>
       </c>
       <c r="C164" s="0" t="inlineStr">
@@ -9889,7 +9889,7 @@
       </c>
       <c r="G164" s="0" t="inlineStr">
         <is>
-          <t>2026-08-21 22:29:43</t>
+          <t>2026-08-21 22:53:02</t>
         </is>
       </c>
       <c r="H164" s="0" t="inlineStr">
@@ -9920,11 +9920,11 @@
     </row>
     <row r="165" spans="1:14">
       <c r="A165" s="0">
-        <v>49455301</v>
+        <v>49493126</v>
       </c>
       <c r="B165" s="0" t="inlineStr">
         <is>
-          <t>周开平</t>
+          <t>刘盼昭</t>
         </is>
       </c>
       <c r="C165" s="0" t="inlineStr">
@@ -9949,7 +9949,7 @@
       </c>
       <c r="G165" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 22:46:59</t>
+          <t>2026-08-21 22:44:53</t>
         </is>
       </c>
       <c r="H165" s="0" t="inlineStr">
@@ -9980,11 +9980,11 @@
     </row>
     <row r="166" spans="1:14">
       <c r="A166" s="0">
-        <v>49432023</v>
+        <v>49492499</v>
       </c>
       <c r="B166" s="0" t="inlineStr">
         <is>
-          <t>花生米</t>
+          <t>红霞</t>
         </is>
       </c>
       <c r="C166" s="0" t="inlineStr">
@@ -10009,7 +10009,7 @@
       </c>
       <c r="G166" s="0" t="inlineStr">
         <is>
-          <t>2026-08-20 11:55:45</t>
+          <t>2026-08-21 22:29:43</t>
         </is>
       </c>
       <c r="H166" s="0" t="inlineStr">
@@ -10040,11 +10040,11 @@
     </row>
     <row r="167" spans="1:14">
       <c r="A167" s="0">
-        <v>49415939</v>
+        <v>49455301</v>
       </c>
       <c r="B167" s="0" t="inlineStr">
         <is>
-          <t>杨梅芳</t>
+          <t>周开平</t>
         </is>
       </c>
       <c r="C167" s="0" t="inlineStr">
@@ -10069,7 +10069,7 @@
       </c>
       <c r="G167" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:58</t>
+          <t>2026-08-20 22:46:59</t>
         </is>
       </c>
       <c r="H167" s="0" t="inlineStr">
@@ -10079,17 +10079,17 @@
       </c>
       <c r="I167" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J167" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K167" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L167" s="0" t="inlineStr">
@@ -10100,11 +10100,11 @@
     </row>
     <row r="168" spans="1:14">
       <c r="A168" s="0">
-        <v>49415918</v>
+        <v>49432023</v>
       </c>
       <c r="B168" s="0" t="inlineStr">
         <is>
-          <t>心语无言</t>
+          <t>花生米</t>
         </is>
       </c>
       <c r="C168" s="0" t="inlineStr">
@@ -10129,7 +10129,7 @@
       </c>
       <c r="G168" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:24</t>
+          <t>2026-08-20 11:55:45</t>
         </is>
       </c>
       <c r="H168" s="0" t="inlineStr">
@@ -10139,17 +10139,17 @@
       </c>
       <c r="I168" s="0" t="inlineStr">
         <is>
-          <t>黄老师-抖音01</t>
+          <t>黄老师-视频号01</t>
         </is>
       </c>
       <c r="J168" s="0" t="inlineStr">
         <is>
-          <t>安迪钢琴-多个点击报名-0元</t>
+          <t>安迪钢琴-获客助手专用</t>
         </is>
       </c>
       <c r="K168" s="0" t="inlineStr">
         <is>
-          <t>微信支付</t>
+          <t>获客助手加好友</t>
         </is>
       </c>
       <c r="L168" s="0" t="inlineStr">
@@ -10160,11 +10160,11 @@
     </row>
     <row r="169" spans="1:14">
       <c r="A169" s="0">
-        <v>49415913</v>
+        <v>49415939</v>
       </c>
       <c r="B169" s="0" t="inlineStr">
         <is>
-          <t>安好</t>
+          <t>杨梅芳</t>
         </is>
       </c>
       <c r="C169" s="0" t="inlineStr">
@@ -10189,7 +10189,7 @@
       </c>
       <c r="G169" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:48:18</t>
+          <t>2026-08-19 22:48:58</t>
         </is>
       </c>
       <c r="H169" s="0" t="inlineStr">
@@ -10220,11 +10220,11 @@
     </row>
     <row r="170" spans="1:14">
       <c r="A170" s="0">
-        <v>49415890</v>
+        <v>49415918</v>
       </c>
       <c r="B170" s="0" t="inlineStr">
         <is>
-          <t>雨夜聆风</t>
+          <t>心语无言</t>
         </is>
       </c>
       <c r="C170" s="0" t="inlineStr">
@@ -10249,7 +10249,7 @@
       </c>
       <c r="G170" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:56</t>
+          <t>2026-08-19 22:48:24</t>
         </is>
       </c>
       <c r="H170" s="0" t="inlineStr">
@@ -10275,21 +10275,16 @@
       <c r="L170" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
-        </is>
-      </c>
-      <c r="N170" s="0" t="inlineStr">
-        <is>
-          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="171" spans="1:14">
       <c r="A171" s="0">
-        <v>49415874</v>
+        <v>49415913</v>
       </c>
       <c r="B171" s="0" t="inlineStr">
         <is>
-          <t>飘</t>
+          <t>安好</t>
         </is>
       </c>
       <c r="C171" s="0" t="inlineStr">
@@ -10314,7 +10309,7 @@
       </c>
       <c r="G171" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:40</t>
+          <t>2026-08-19 22:48:18</t>
         </is>
       </c>
       <c r="H171" s="0" t="inlineStr">
@@ -10345,11 +10340,11 @@
     </row>
     <row r="172" spans="1:14">
       <c r="A172" s="0">
-        <v>49415871</v>
+        <v>49415890</v>
       </c>
       <c r="B172" s="0" t="inlineStr">
         <is>
-          <t>庆</t>
+          <t>雨夜聆风</t>
         </is>
       </c>
       <c r="C172" s="0" t="inlineStr">
@@ -10374,7 +10369,7 @@
       </c>
       <c r="G172" s="0" t="inlineStr">
         <is>
-          <t>2026-08-19 22:47:36</t>
+          <t>2026-08-19 22:47:56</t>
         </is>
       </c>
       <c r="H172" s="0" t="inlineStr">
@@ -10400,64 +10395,189 @@
       <c r="L172" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
+        </is>
+      </c>
+      <c r="N172" s="0" t="inlineStr">
+        <is>
+          <t>宜春</t>
         </is>
       </c>
     </row>
     <row r="173" spans="1:14">
       <c r="A173" s="0">
+        <v>49415874</v>
+      </c>
+      <c r="B173" s="0" t="inlineStr">
+        <is>
+          <t>飘</t>
+        </is>
+      </c>
+      <c r="C173" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D173" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E173" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F173" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G173" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:40</t>
+        </is>
+      </c>
+      <c r="H173" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I173" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J173" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K173" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L173" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" spans="1:14">
+      <c r="A174" s="0">
+        <v>49415871</v>
+      </c>
+      <c r="B174" s="0" t="inlineStr">
+        <is>
+          <t>庆</t>
+        </is>
+      </c>
+      <c r="C174" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D174" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E174" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F174" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G174" s="0" t="inlineStr">
+        <is>
+          <t>2026-08-19 22:47:36</t>
+        </is>
+      </c>
+      <c r="H174" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I174" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J174" s="0" t="inlineStr">
+        <is>
+          <t>安迪钢琴-多个点击报名-0元</t>
+        </is>
+      </c>
+      <c r="K174" s="0" t="inlineStr">
+        <is>
+          <t>微信支付</t>
+        </is>
+      </c>
+      <c r="L174" s="0" t="inlineStr">
+        <is>
+          <t>已完成</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" spans="1:14">
+      <c r="A175" s="0">
         <v>49415867</v>
       </c>
-      <c r="B173" s="0" t="inlineStr">
+      <c r="B175" s="0" t="inlineStr">
         <is>
           <t>HYQ</t>
         </is>
       </c>
-      <c r="C173" s="0" t="inlineStr">
-        <is>
-          <t>6天0基础钢琴入门课</t>
-        </is>
-      </c>
-      <c r="D173" s="0" t="inlineStr">
-        <is>
-          <t>训练营</t>
-        </is>
-      </c>
-      <c r="E173" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="F173" s="0" t="inlineStr">
-        <is>
-          <t>￥0</t>
-        </is>
-      </c>
-      <c r="G173" s="0" t="inlineStr">
+      <c r="C175" s="0" t="inlineStr">
+        <is>
+          <t>6天0基础钢琴入门课</t>
+        </is>
+      </c>
+      <c r="D175" s="0" t="inlineStr">
+        <is>
+          <t>训练营</t>
+        </is>
+      </c>
+      <c r="E175" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="F175" s="0" t="inlineStr">
+        <is>
+          <t>￥0</t>
+        </is>
+      </c>
+      <c r="G175" s="0" t="inlineStr">
         <is>
           <t>2026-08-19 22:47:33</t>
         </is>
       </c>
-      <c r="H173" s="0" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I173" s="0" t="inlineStr">
-        <is>
-          <t>黄老师-抖音01</t>
-        </is>
-      </c>
-      <c r="J173" s="0" t="inlineStr">
+      <c r="H175" s="0" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I175" s="0" t="inlineStr">
+        <is>
+          <t>黄老师-抖音01</t>
+        </is>
+      </c>
+      <c r="J175" s="0" t="inlineStr">
         <is>
           <t>安迪钢琴-多个点击报名-0元</t>
         </is>
       </c>
-      <c r="K173" s="0" t="inlineStr">
+      <c r="K175" s="0" t="inlineStr">
         <is>
           <t>微信支付</t>
         </is>
       </c>
-      <c r="L173" s="0" t="inlineStr">
+      <c r="L175" s="0" t="inlineStr">
         <is>
           <t>已完成</t>
         </is>

</xml_diff>